<commit_message>
Synka blankett_forvaltarkunskap_nnk.xlsx med v1.6 (radgruppering per objekt)
Rent layout-/UX-ändring, ingen ny personuppgift - synkat direkt enligt
tidigare överenskommelse.
</commit_message>
<xml_diff>
--- a/blanketter/blankett_forvaltarkunskap_nnk.xlsx
+++ b/blanketter/blankett_forvaltarkunskap_nnk.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C32"/>
+  <dimension ref="B2:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -741,7 +741,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.5, 2026-08-27</t>
+          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.6, 2026-08-27</t>
         </is>
       </c>
     </row>
@@ -881,113 +881,125 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="19" ht="70" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>10.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Nytt sedan version 1.6: rader grupperade per objekt. Ett objekt med flera naturtyper visar bara sin första rad — klicka på [+] i vänstermarginalen (eller Disposition-fliken i Excel) för att fälla ut de övriga naturtyprader som hör till samma objekt. Gör bara blanketten kortare att bläddra i, ändrar ingen data. Om du filtrerar (punkt 1): fäll ut grupperna innan du filtrerar, annars kan dolda naturtyprader missas i urvalet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Tre regler att ha med sig i samtalet</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="42" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>En igenvuxen äng är fortfarande en äng. Om orsaken är utebliven skötsel ska livsmiljötypen stå kvar och tillståndet sättas till Icke gott — inte klassas om till annan naturtyp. (Lathunden, "Vad kan vi ändra på?")</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Kunskap som funnits men aldrig registrerats är en Komplettering, inte en Faktisk förändring. Det avgör om länet rapporterar in en arealförändring som aldrig hänt. (Handledningen 5.4)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Kunskap som funnits men aldrig registrerats är en Komplettering, inte en Faktisk förändring. Det avgör om länet rapporterar in en arealförändring som aldrig hänt. (Handledningen 5.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Fråga alltid efter årtal. Utan datering går FAQ fråga 4:s krav på "hur aktuell bedömningen är" inte att besvara.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Flikar</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Blankett</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>628 rader, en per objekt × livsmiljötyp. Sorterad med prioritet 1 först.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Åtgärdas-ytor</t>
+          <t>Blankett</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>De 141 ytor med karteringsstatus 5, per objekt och livsmiljötyp.</t>
+          <t>628 rader, en per objekt × livsmiljötyp. Sorterad med prioritet 1 först.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Kodlistor</t>
+          <t>Åtgärdas-ytor</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Tillåtna värden. Källa till rullistorna — redigera inte.</t>
+          <t>De 141 ytor med karteringsstatus 5, per objekt och livsmiljötyp.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>Kodlistor</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Tillåtna värden. Källa till rullistorna — redigera inte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="14" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
           <t>Fältmappning</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Vilken blankettkolumn som hamnar i vilket fält i granskningslagret och NNK.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Källor</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="2" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Förifylld areal och objektsurval: NNK-statistik per Natura 2000-område D-län, uttag 2026-01-20 (Naturvårdsverket). Åtgärdas-ytorna: NNK-lagrets attributtabell, uttag från ArcGIS Pro 2026-08-17. Kodvärden: Handledning för NNK 2026-07-03 samt Lathund granskning WebbGIS-KartLitS 2026-07-10.</t>
         </is>
@@ -996,14 +1008,14 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B21:C21"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B20:C20"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B9:C9"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -1023,7 +1035,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF1F3864"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y630"/>
@@ -1357,7 +1369,7 @@
       <c r="X3" s="15" t="n"/>
       <c r="Y3" s="15" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" hidden="1" outlineLevel="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1418,7 +1430,7 @@
       <c r="X4" s="15" t="n"/>
       <c r="Y4" s="15" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" hidden="1" outlineLevel="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1479,7 +1491,7 @@
       <c r="X5" s="15" t="n"/>
       <c r="Y5" s="15" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" hidden="1" outlineLevel="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1540,7 +1552,7 @@
       <c r="X6" s="15" t="n"/>
       <c r="Y6" s="15" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" hidden="1" outlineLevel="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1601,7 +1613,7 @@
       <c r="X7" s="15" t="n"/>
       <c r="Y7" s="15" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" hidden="1" outlineLevel="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1662,7 +1674,7 @@
       <c r="X8" s="15" t="n"/>
       <c r="Y8" s="15" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" hidden="1" outlineLevel="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1723,7 +1735,7 @@
       <c r="X9" s="15" t="n"/>
       <c r="Y9" s="15" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" hidden="1" outlineLevel="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1784,7 +1796,7 @@
       <c r="X10" s="15" t="n"/>
       <c r="Y10" s="15" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" hidden="1" outlineLevel="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1845,7 +1857,7 @@
       <c r="X11" s="15" t="n"/>
       <c r="Y11" s="15" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" hidden="1" outlineLevel="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1906,7 +1918,7 @@
       <c r="X12" s="15" t="n"/>
       <c r="Y12" s="15" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" hidden="1" outlineLevel="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -1967,7 +1979,7 @@
       <c r="X13" s="15" t="n"/>
       <c r="Y13" s="15" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" hidden="1" outlineLevel="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2028,7 +2040,7 @@
       <c r="X14" s="15" t="n"/>
       <c r="Y14" s="15" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2089,7 +2101,7 @@
       <c r="X15" s="15" t="n"/>
       <c r="Y15" s="15" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" hidden="1" outlineLevel="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2150,7 +2162,7 @@
       <c r="X16" s="15" t="n"/>
       <c r="Y16" s="15" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" hidden="1" outlineLevel="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2211,7 +2223,7 @@
       <c r="X17" s="15" t="n"/>
       <c r="Y17" s="15" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" hidden="1" outlineLevel="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2272,7 +2284,7 @@
       <c r="X18" s="15" t="n"/>
       <c r="Y18" s="15" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" hidden="1" outlineLevel="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2333,7 +2345,7 @@
       <c r="X19" s="15" t="n"/>
       <c r="Y19" s="15" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" hidden="1" outlineLevel="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2394,7 +2406,7 @@
       <c r="X20" s="15" t="n"/>
       <c r="Y20" s="15" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" hidden="1" outlineLevel="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2455,7 +2467,7 @@
       <c r="X21" s="15" t="n"/>
       <c r="Y21" s="15" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" hidden="1" outlineLevel="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2516,7 +2528,7 @@
       <c r="X22" s="15" t="n"/>
       <c r="Y22" s="15" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" hidden="1" outlineLevel="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2577,7 +2589,7 @@
       <c r="X23" s="15" t="n"/>
       <c r="Y23" s="15" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" hidden="1" outlineLevel="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2638,7 +2650,7 @@
       <c r="X24" s="15" t="n"/>
       <c r="Y24" s="15" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" hidden="1" outlineLevel="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2699,7 +2711,7 @@
       <c r="X25" s="15" t="n"/>
       <c r="Y25" s="15" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" hidden="1" outlineLevel="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2760,7 +2772,7 @@
       <c r="X26" s="15" t="n"/>
       <c r="Y26" s="15" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" hidden="1" outlineLevel="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2821,7 +2833,7 @@
       <c r="X27" s="15" t="n"/>
       <c r="Y27" s="15" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" hidden="1" outlineLevel="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -2882,7 +2894,7 @@
       <c r="X28" s="15" t="n"/>
       <c r="Y28" s="15" t="n"/>
     </row>
-    <row r="29">
+    <row r="29" hidden="1" outlineLevel="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3008,7 +3020,7 @@
       <c r="X30" s="15" t="n"/>
       <c r="Y30" s="15" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" hidden="1" outlineLevel="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3073,7 +3085,7 @@
       <c r="X31" s="15" t="n"/>
       <c r="Y31" s="15" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" hidden="1" outlineLevel="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3138,7 +3150,7 @@
       <c r="X32" s="15" t="n"/>
       <c r="Y32" s="15" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" hidden="1" outlineLevel="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3203,7 +3215,7 @@
       <c r="X33" s="15" t="n"/>
       <c r="Y33" s="15" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" hidden="1" outlineLevel="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3268,7 +3280,7 @@
       <c r="X34" s="15" t="n"/>
       <c r="Y34" s="15" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" hidden="1" outlineLevel="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3333,7 +3345,7 @@
       <c r="X35" s="15" t="n"/>
       <c r="Y35" s="15" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" hidden="1" outlineLevel="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3398,7 +3410,7 @@
       <c r="X36" s="15" t="n"/>
       <c r="Y36" s="15" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" hidden="1" outlineLevel="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3463,7 +3475,7 @@
       <c r="X37" s="15" t="n"/>
       <c r="Y37" s="15" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" hidden="1" outlineLevel="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3528,7 +3540,7 @@
       <c r="X38" s="15" t="n"/>
       <c r="Y38" s="15" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" hidden="1" outlineLevel="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3593,7 +3605,7 @@
       <c r="X39" s="15" t="n"/>
       <c r="Y39" s="15" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" hidden="1" outlineLevel="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3658,7 +3670,7 @@
       <c r="X40" s="15" t="n"/>
       <c r="Y40" s="15" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" hidden="1" outlineLevel="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3723,7 +3735,7 @@
       <c r="X41" s="15" t="n"/>
       <c r="Y41" s="15" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" hidden="1" outlineLevel="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3788,7 +3800,7 @@
       <c r="X42" s="15" t="n"/>
       <c r="Y42" s="15" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" hidden="1" outlineLevel="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3853,7 +3865,7 @@
       <c r="X43" s="15" t="n"/>
       <c r="Y43" s="15" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" hidden="1" outlineLevel="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3918,7 +3930,7 @@
       <c r="X44" s="15" t="n"/>
       <c r="Y44" s="15" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" hidden="1" outlineLevel="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -3983,7 +3995,7 @@
       <c r="X45" s="15" t="n"/>
       <c r="Y45" s="15" t="n"/>
     </row>
-    <row r="46">
+    <row r="46" hidden="1" outlineLevel="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4048,7 +4060,7 @@
       <c r="X46" s="15" t="n"/>
       <c r="Y46" s="15" t="n"/>
     </row>
-    <row r="47">
+    <row r="47" hidden="1" outlineLevel="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4182,7 +4194,7 @@
       <c r="X48" s="15" t="n"/>
       <c r="Y48" s="15" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" hidden="1" outlineLevel="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4251,7 +4263,7 @@
       <c r="X49" s="15" t="n"/>
       <c r="Y49" s="15" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" hidden="1" outlineLevel="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4320,7 +4332,7 @@
       <c r="X50" s="15" t="n"/>
       <c r="Y50" s="15" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" hidden="1" outlineLevel="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4389,7 +4401,7 @@
       <c r="X51" s="15" t="n"/>
       <c r="Y51" s="15" t="n"/>
     </row>
-    <row r="52">
+    <row r="52" hidden="1" outlineLevel="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4458,7 +4470,7 @@
       <c r="X52" s="15" t="n"/>
       <c r="Y52" s="15" t="n"/>
     </row>
-    <row r="53">
+    <row r="53" hidden="1" outlineLevel="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4527,7 +4539,7 @@
       <c r="X53" s="15" t="n"/>
       <c r="Y53" s="15" t="n"/>
     </row>
-    <row r="54">
+    <row r="54" hidden="1" outlineLevel="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4596,7 +4608,7 @@
       <c r="X54" s="15" t="n"/>
       <c r="Y54" s="15" t="n"/>
     </row>
-    <row r="55">
+    <row r="55" hidden="1" outlineLevel="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4665,7 +4677,7 @@
       <c r="X55" s="15" t="n"/>
       <c r="Y55" s="15" t="n"/>
     </row>
-    <row r="56">
+    <row r="56" hidden="1" outlineLevel="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4734,7 +4746,7 @@
       <c r="X56" s="15" t="n"/>
       <c r="Y56" s="15" t="n"/>
     </row>
-    <row r="57">
+    <row r="57" hidden="1" outlineLevel="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4803,7 +4815,7 @@
       <c r="X57" s="15" t="n"/>
       <c r="Y57" s="15" t="n"/>
     </row>
-    <row r="58">
+    <row r="58" hidden="1" outlineLevel="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4872,7 +4884,7 @@
       <c r="X58" s="15" t="n"/>
       <c r="Y58" s="15" t="n"/>
     </row>
-    <row r="59">
+    <row r="59" hidden="1" outlineLevel="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -4941,7 +4953,7 @@
       <c r="X59" s="15" t="n"/>
       <c r="Y59" s="15" t="n"/>
     </row>
-    <row r="60">
+    <row r="60" hidden="1" outlineLevel="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5010,7 +5022,7 @@
       <c r="X60" s="15" t="n"/>
       <c r="Y60" s="15" t="n"/>
     </row>
-    <row r="61">
+    <row r="61" hidden="1" outlineLevel="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5144,7 +5156,7 @@
       <c r="X62" s="15" t="n"/>
       <c r="Y62" s="15" t="n"/>
     </row>
-    <row r="63">
+    <row r="63" hidden="1" outlineLevel="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5209,7 +5221,7 @@
       <c r="X63" s="15" t="n"/>
       <c r="Y63" s="15" t="n"/>
     </row>
-    <row r="64">
+    <row r="64" hidden="1" outlineLevel="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5274,7 +5286,7 @@
       <c r="X64" s="15" t="n"/>
       <c r="Y64" s="15" t="n"/>
     </row>
-    <row r="65">
+    <row r="65" hidden="1" outlineLevel="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5339,7 +5351,7 @@
       <c r="X65" s="15" t="n"/>
       <c r="Y65" s="15" t="n"/>
     </row>
-    <row r="66">
+    <row r="66" hidden="1" outlineLevel="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5404,7 +5416,7 @@
       <c r="X66" s="15" t="n"/>
       <c r="Y66" s="15" t="n"/>
     </row>
-    <row r="67">
+    <row r="67" hidden="1" outlineLevel="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5469,7 +5481,7 @@
       <c r="X67" s="15" t="n"/>
       <c r="Y67" s="15" t="n"/>
     </row>
-    <row r="68">
+    <row r="68" hidden="1" outlineLevel="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5534,7 +5546,7 @@
       <c r="X68" s="15" t="n"/>
       <c r="Y68" s="15" t="n"/>
     </row>
-    <row r="69">
+    <row r="69" hidden="1" outlineLevel="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5599,7 +5611,7 @@
       <c r="X69" s="15" t="n"/>
       <c r="Y69" s="15" t="n"/>
     </row>
-    <row r="70">
+    <row r="70" hidden="1" outlineLevel="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5664,7 +5676,7 @@
       <c r="X70" s="15" t="n"/>
       <c r="Y70" s="15" t="n"/>
     </row>
-    <row r="71">
+    <row r="71" hidden="1" outlineLevel="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5729,7 +5741,7 @@
       <c r="X71" s="15" t="n"/>
       <c r="Y71" s="15" t="n"/>
     </row>
-    <row r="72">
+    <row r="72" hidden="1" outlineLevel="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5794,7 +5806,7 @@
       <c r="X72" s="15" t="n"/>
       <c r="Y72" s="15" t="n"/>
     </row>
-    <row r="73">
+    <row r="73" hidden="1" outlineLevel="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5859,7 +5871,7 @@
       <c r="X73" s="15" t="n"/>
       <c r="Y73" s="15" t="n"/>
     </row>
-    <row r="74">
+    <row r="74" hidden="1" outlineLevel="1">
       <c r="A74" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5924,7 +5936,7 @@
       <c r="X74" s="15" t="n"/>
       <c r="Y74" s="15" t="n"/>
     </row>
-    <row r="75">
+    <row r="75" hidden="1" outlineLevel="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -5989,7 +6001,7 @@
       <c r="X75" s="15" t="n"/>
       <c r="Y75" s="15" t="n"/>
     </row>
-    <row r="76">
+    <row r="76" hidden="1" outlineLevel="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6054,7 +6066,7 @@
       <c r="X76" s="15" t="n"/>
       <c r="Y76" s="15" t="n"/>
     </row>
-    <row r="77">
+    <row r="77" hidden="1" outlineLevel="1">
       <c r="A77" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6119,7 +6131,7 @@
       <c r="X77" s="15" t="n"/>
       <c r="Y77" s="15" t="n"/>
     </row>
-    <row r="78">
+    <row r="78" hidden="1" outlineLevel="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6184,7 +6196,7 @@
       <c r="X78" s="15" t="n"/>
       <c r="Y78" s="15" t="n"/>
     </row>
-    <row r="79">
+    <row r="79" hidden="1" outlineLevel="1">
       <c r="A79" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6314,7 +6326,7 @@
       <c r="X80" s="15" t="n"/>
       <c r="Y80" s="15" t="n"/>
     </row>
-    <row r="81">
+    <row r="81" hidden="1" outlineLevel="1">
       <c r="A81" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6379,7 +6391,7 @@
       <c r="X81" s="15" t="n"/>
       <c r="Y81" s="15" t="n"/>
     </row>
-    <row r="82">
+    <row r="82" hidden="1" outlineLevel="1">
       <c r="A82" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6444,7 +6456,7 @@
       <c r="X82" s="15" t="n"/>
       <c r="Y82" s="15" t="n"/>
     </row>
-    <row r="83">
+    <row r="83" hidden="1" outlineLevel="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6509,7 +6521,7 @@
       <c r="X83" s="15" t="n"/>
       <c r="Y83" s="15" t="n"/>
     </row>
-    <row r="84">
+    <row r="84" hidden="1" outlineLevel="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6574,7 +6586,7 @@
       <c r="X84" s="15" t="n"/>
       <c r="Y84" s="15" t="n"/>
     </row>
-    <row r="85">
+    <row r="85" hidden="1" outlineLevel="1">
       <c r="A85" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6639,7 +6651,7 @@
       <c r="X85" s="15" t="n"/>
       <c r="Y85" s="15" t="n"/>
     </row>
-    <row r="86">
+    <row r="86" hidden="1" outlineLevel="1">
       <c r="A86" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6704,7 +6716,7 @@
       <c r="X86" s="15" t="n"/>
       <c r="Y86" s="15" t="n"/>
     </row>
-    <row r="87">
+    <row r="87" hidden="1" outlineLevel="1">
       <c r="A87" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6834,7 +6846,7 @@
       <c r="X88" s="15" t="n"/>
       <c r="Y88" s="15" t="n"/>
     </row>
-    <row r="89">
+    <row r="89" hidden="1" outlineLevel="1">
       <c r="A89" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6899,7 +6911,7 @@
       <c r="X89" s="15" t="n"/>
       <c r="Y89" s="15" t="n"/>
     </row>
-    <row r="90">
+    <row r="90" hidden="1" outlineLevel="1">
       <c r="A90" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -6964,7 +6976,7 @@
       <c r="X90" s="15" t="n"/>
       <c r="Y90" s="15" t="n"/>
     </row>
-    <row r="91">
+    <row r="91" hidden="1" outlineLevel="1">
       <c r="A91" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7029,7 +7041,7 @@
       <c r="X91" s="15" t="n"/>
       <c r="Y91" s="15" t="n"/>
     </row>
-    <row r="92">
+    <row r="92" hidden="1" outlineLevel="1">
       <c r="A92" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7094,7 +7106,7 @@
       <c r="X92" s="15" t="n"/>
       <c r="Y92" s="15" t="n"/>
     </row>
-    <row r="93">
+    <row r="93" hidden="1" outlineLevel="1">
       <c r="A93" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7159,7 +7171,7 @@
       <c r="X93" s="15" t="n"/>
       <c r="Y93" s="15" t="n"/>
     </row>
-    <row r="94">
+    <row r="94" hidden="1" outlineLevel="1">
       <c r="A94" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7224,7 +7236,7 @@
       <c r="X94" s="15" t="n"/>
       <c r="Y94" s="15" t="n"/>
     </row>
-    <row r="95">
+    <row r="95" hidden="1" outlineLevel="1">
       <c r="A95" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7289,7 +7301,7 @@
       <c r="X95" s="15" t="n"/>
       <c r="Y95" s="15" t="n"/>
     </row>
-    <row r="96">
+    <row r="96" hidden="1" outlineLevel="1">
       <c r="A96" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7354,7 +7366,7 @@
       <c r="X96" s="15" t="n"/>
       <c r="Y96" s="15" t="n"/>
     </row>
-    <row r="97">
+    <row r="97" hidden="1" outlineLevel="1">
       <c r="A97" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7419,7 +7431,7 @@
       <c r="X97" s="15" t="n"/>
       <c r="Y97" s="15" t="n"/>
     </row>
-    <row r="98">
+    <row r="98" hidden="1" outlineLevel="1">
       <c r="A98" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7484,7 +7496,7 @@
       <c r="X98" s="15" t="n"/>
       <c r="Y98" s="15" t="n"/>
     </row>
-    <row r="99">
+    <row r="99" hidden="1" outlineLevel="1">
       <c r="A99" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7614,7 +7626,7 @@
       <c r="X100" s="15" t="n"/>
       <c r="Y100" s="15" t="n"/>
     </row>
-    <row r="101">
+    <row r="101" hidden="1" outlineLevel="1">
       <c r="A101" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7679,7 +7691,7 @@
       <c r="X101" s="15" t="n"/>
       <c r="Y101" s="15" t="n"/>
     </row>
-    <row r="102">
+    <row r="102" hidden="1" outlineLevel="1">
       <c r="A102" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7813,7 +7825,7 @@
       <c r="X103" s="15" t="n"/>
       <c r="Y103" s="15" t="n"/>
     </row>
-    <row r="104">
+    <row r="104" hidden="1" outlineLevel="1">
       <c r="A104" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7882,7 +7894,7 @@
       <c r="X104" s="15" t="n"/>
       <c r="Y104" s="15" t="n"/>
     </row>
-    <row r="105">
+    <row r="105" hidden="1" outlineLevel="1">
       <c r="A105" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -7951,7 +7963,7 @@
       <c r="X105" s="15" t="n"/>
       <c r="Y105" s="15" t="n"/>
     </row>
-    <row r="106">
+    <row r="106" hidden="1" outlineLevel="1">
       <c r="A106" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8020,7 +8032,7 @@
       <c r="X106" s="15" t="n"/>
       <c r="Y106" s="15" t="n"/>
     </row>
-    <row r="107">
+    <row r="107" hidden="1" outlineLevel="1">
       <c r="A107" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8089,7 +8101,7 @@
       <c r="X107" s="15" t="n"/>
       <c r="Y107" s="15" t="n"/>
     </row>
-    <row r="108">
+    <row r="108" hidden="1" outlineLevel="1">
       <c r="A108" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8227,7 +8239,7 @@
       <c r="X109" s="15" t="n"/>
       <c r="Y109" s="15" t="n"/>
     </row>
-    <row r="110">
+    <row r="110" hidden="1" outlineLevel="1">
       <c r="A110" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8296,7 +8308,7 @@
       <c r="X110" s="15" t="n"/>
       <c r="Y110" s="15" t="n"/>
     </row>
-    <row r="111">
+    <row r="111" hidden="1" outlineLevel="1">
       <c r="A111" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8365,7 +8377,7 @@
       <c r="X111" s="15" t="n"/>
       <c r="Y111" s="15" t="n"/>
     </row>
-    <row r="112">
+    <row r="112" hidden="1" outlineLevel="1">
       <c r="A112" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8434,7 +8446,7 @@
       <c r="X112" s="15" t="n"/>
       <c r="Y112" s="15" t="n"/>
     </row>
-    <row r="113">
+    <row r="113" hidden="1" outlineLevel="1">
       <c r="A113" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8503,7 +8515,7 @@
       <c r="X113" s="15" t="n"/>
       <c r="Y113" s="15" t="n"/>
     </row>
-    <row r="114">
+    <row r="114" hidden="1" outlineLevel="1">
       <c r="A114" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8572,7 +8584,7 @@
       <c r="X114" s="15" t="n"/>
       <c r="Y114" s="15" t="n"/>
     </row>
-    <row r="115">
+    <row r="115" hidden="1" outlineLevel="1">
       <c r="A115" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8641,7 +8653,7 @@
       <c r="X115" s="15" t="n"/>
       <c r="Y115" s="15" t="n"/>
     </row>
-    <row r="116">
+    <row r="116" hidden="1" outlineLevel="1">
       <c r="A116" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8710,7 +8722,7 @@
       <c r="X116" s="15" t="n"/>
       <c r="Y116" s="15" t="n"/>
     </row>
-    <row r="117">
+    <row r="117" hidden="1" outlineLevel="1">
       <c r="A117" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8779,7 +8791,7 @@
       <c r="X117" s="15" t="n"/>
       <c r="Y117" s="15" t="n"/>
     </row>
-    <row r="118">
+    <row r="118" hidden="1" outlineLevel="1">
       <c r="A118" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8848,7 +8860,7 @@
       <c r="X118" s="15" t="n"/>
       <c r="Y118" s="15" t="n"/>
     </row>
-    <row r="119">
+    <row r="119" hidden="1" outlineLevel="1">
       <c r="A119" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8917,7 +8929,7 @@
       <c r="X119" s="15" t="n"/>
       <c r="Y119" s="15" t="n"/>
     </row>
-    <row r="120">
+    <row r="120" hidden="1" outlineLevel="1">
       <c r="A120" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -8986,7 +8998,7 @@
       <c r="X120" s="15" t="n"/>
       <c r="Y120" s="15" t="n"/>
     </row>
-    <row r="121">
+    <row r="121" hidden="1" outlineLevel="1">
       <c r="A121" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9120,7 +9132,7 @@
       <c r="X122" s="15" t="n"/>
       <c r="Y122" s="15" t="n"/>
     </row>
-    <row r="123">
+    <row r="123" hidden="1" outlineLevel="1">
       <c r="A123" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9185,7 +9197,7 @@
       <c r="X123" s="15" t="n"/>
       <c r="Y123" s="15" t="n"/>
     </row>
-    <row r="124">
+    <row r="124" hidden="1" outlineLevel="1">
       <c r="A124" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9250,7 +9262,7 @@
       <c r="X124" s="15" t="n"/>
       <c r="Y124" s="15" t="n"/>
     </row>
-    <row r="125">
+    <row r="125" hidden="1" outlineLevel="1">
       <c r="A125" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9315,7 +9327,7 @@
       <c r="X125" s="15" t="n"/>
       <c r="Y125" s="15" t="n"/>
     </row>
-    <row r="126">
+    <row r="126" hidden="1" outlineLevel="1">
       <c r="A126" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9514,7 +9526,7 @@
       <c r="X128" s="15" t="n"/>
       <c r="Y128" s="15" t="n"/>
     </row>
-    <row r="129">
+    <row r="129" hidden="1" outlineLevel="1">
       <c r="A129" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9583,7 +9595,7 @@
       <c r="X129" s="15" t="n"/>
       <c r="Y129" s="15" t="n"/>
     </row>
-    <row r="130">
+    <row r="130" hidden="1" outlineLevel="1">
       <c r="A130" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9652,7 +9664,7 @@
       <c r="X130" s="15" t="n"/>
       <c r="Y130" s="15" t="n"/>
     </row>
-    <row r="131">
+    <row r="131" hidden="1" outlineLevel="1">
       <c r="A131" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9721,7 +9733,7 @@
       <c r="X131" s="15" t="n"/>
       <c r="Y131" s="15" t="n"/>
     </row>
-    <row r="132">
+    <row r="132" hidden="1" outlineLevel="1">
       <c r="A132" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9790,7 +9802,7 @@
       <c r="X132" s="15" t="n"/>
       <c r="Y132" s="15" t="n"/>
     </row>
-    <row r="133">
+    <row r="133" hidden="1" outlineLevel="1">
       <c r="A133" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9859,7 +9871,7 @@
       <c r="X133" s="15" t="n"/>
       <c r="Y133" s="15" t="n"/>
     </row>
-    <row r="134">
+    <row r="134" hidden="1" outlineLevel="1">
       <c r="A134" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9928,7 +9940,7 @@
       <c r="X134" s="15" t="n"/>
       <c r="Y134" s="15" t="n"/>
     </row>
-    <row r="135">
+    <row r="135" hidden="1" outlineLevel="1">
       <c r="A135" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9997,7 +10009,7 @@
       <c r="X135" s="15" t="n"/>
       <c r="Y135" s="15" t="n"/>
     </row>
-    <row r="136">
+    <row r="136" hidden="1" outlineLevel="1">
       <c r="A136" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10131,7 +10143,7 @@
       <c r="X137" s="15" t="n"/>
       <c r="Y137" s="15" t="n"/>
     </row>
-    <row r="138">
+    <row r="138" hidden="1" outlineLevel="1">
       <c r="A138" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10196,7 +10208,7 @@
       <c r="X138" s="15" t="n"/>
       <c r="Y138" s="15" t="n"/>
     </row>
-    <row r="139">
+    <row r="139" hidden="1" outlineLevel="1">
       <c r="A139" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10261,7 +10273,7 @@
       <c r="X139" s="15" t="n"/>
       <c r="Y139" s="15" t="n"/>
     </row>
-    <row r="140">
+    <row r="140" hidden="1" outlineLevel="1">
       <c r="A140" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10395,7 +10407,7 @@
       <c r="X141" s="15" t="n"/>
       <c r="Y141" s="15" t="n"/>
     </row>
-    <row r="142">
+    <row r="142" hidden="1" outlineLevel="1">
       <c r="A142" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10464,7 +10476,7 @@
       <c r="X142" s="15" t="n"/>
       <c r="Y142" s="15" t="n"/>
     </row>
-    <row r="143">
+    <row r="143" hidden="1" outlineLevel="1">
       <c r="A143" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10533,7 +10545,7 @@
       <c r="X143" s="15" t="n"/>
       <c r="Y143" s="15" t="n"/>
     </row>
-    <row r="144">
+    <row r="144" hidden="1" outlineLevel="1">
       <c r="A144" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10602,7 +10614,7 @@
       <c r="X144" s="15" t="n"/>
       <c r="Y144" s="15" t="n"/>
     </row>
-    <row r="145">
+    <row r="145" hidden="1" outlineLevel="1">
       <c r="A145" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10671,7 +10683,7 @@
       <c r="X145" s="15" t="n"/>
       <c r="Y145" s="15" t="n"/>
     </row>
-    <row r="146">
+    <row r="146" hidden="1" outlineLevel="1">
       <c r="A146" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10740,7 +10752,7 @@
       <c r="X146" s="15" t="n"/>
       <c r="Y146" s="15" t="n"/>
     </row>
-    <row r="147">
+    <row r="147" hidden="1" outlineLevel="1">
       <c r="A147" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10809,7 +10821,7 @@
       <c r="X147" s="15" t="n"/>
       <c r="Y147" s="15" t="n"/>
     </row>
-    <row r="148">
+    <row r="148" hidden="1" outlineLevel="1">
       <c r="A148" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -10943,7 +10955,7 @@
       <c r="X149" s="15" t="n"/>
       <c r="Y149" s="15" t="n"/>
     </row>
-    <row r="150">
+    <row r="150" hidden="1" outlineLevel="1">
       <c r="A150" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11008,7 +11020,7 @@
       <c r="X150" s="15" t="n"/>
       <c r="Y150" s="15" t="n"/>
     </row>
-    <row r="151">
+    <row r="151" hidden="1" outlineLevel="1">
       <c r="A151" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11073,7 +11085,7 @@
       <c r="X151" s="15" t="n"/>
       <c r="Y151" s="15" t="n"/>
     </row>
-    <row r="152">
+    <row r="152" hidden="1" outlineLevel="1">
       <c r="A152" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11138,7 +11150,7 @@
       <c r="X152" s="15" t="n"/>
       <c r="Y152" s="15" t="n"/>
     </row>
-    <row r="153">
+    <row r="153" hidden="1" outlineLevel="1">
       <c r="A153" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11203,7 +11215,7 @@
       <c r="X153" s="15" t="n"/>
       <c r="Y153" s="15" t="n"/>
     </row>
-    <row r="154">
+    <row r="154" hidden="1" outlineLevel="1">
       <c r="A154" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11333,7 +11345,7 @@
       <c r="X155" s="15" t="n"/>
       <c r="Y155" s="15" t="n"/>
     </row>
-    <row r="156">
+    <row r="156" hidden="1" outlineLevel="1">
       <c r="A156" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11398,7 +11410,7 @@
       <c r="X156" s="15" t="n"/>
       <c r="Y156" s="15" t="n"/>
     </row>
-    <row r="157">
+    <row r="157" hidden="1" outlineLevel="1">
       <c r="A157" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11463,7 +11475,7 @@
       <c r="X157" s="15" t="n"/>
       <c r="Y157" s="15" t="n"/>
     </row>
-    <row r="158">
+    <row r="158" hidden="1" outlineLevel="1">
       <c r="A158" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11528,7 +11540,7 @@
       <c r="X158" s="15" t="n"/>
       <c r="Y158" s="15" t="n"/>
     </row>
-    <row r="159">
+    <row r="159" hidden="1" outlineLevel="1">
       <c r="A159" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11662,7 +11674,7 @@
       <c r="X160" s="15" t="n"/>
       <c r="Y160" s="15" t="n"/>
     </row>
-    <row r="161">
+    <row r="161" hidden="1" outlineLevel="1">
       <c r="A161" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11731,7 +11743,7 @@
       <c r="X161" s="15" t="n"/>
       <c r="Y161" s="15" t="n"/>
     </row>
-    <row r="162">
+    <row r="162" hidden="1" outlineLevel="1">
       <c r="A162" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11800,7 +11812,7 @@
       <c r="X162" s="15" t="n"/>
       <c r="Y162" s="15" t="n"/>
     </row>
-    <row r="163">
+    <row r="163" hidden="1" outlineLevel="1">
       <c r="A163" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11869,7 +11881,7 @@
       <c r="X163" s="15" t="n"/>
       <c r="Y163" s="15" t="n"/>
     </row>
-    <row r="164">
+    <row r="164" hidden="1" outlineLevel="1">
       <c r="A164" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -11938,7 +11950,7 @@
       <c r="X164" s="15" t="n"/>
       <c r="Y164" s="15" t="n"/>
     </row>
-    <row r="165">
+    <row r="165" hidden="1" outlineLevel="1">
       <c r="A165" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12007,7 +12019,7 @@
       <c r="X165" s="15" t="n"/>
       <c r="Y165" s="15" t="n"/>
     </row>
-    <row r="166">
+    <row r="166" hidden="1" outlineLevel="1">
       <c r="A166" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12141,7 +12153,7 @@
       <c r="X167" s="15" t="n"/>
       <c r="Y167" s="15" t="n"/>
     </row>
-    <row r="168">
+    <row r="168" hidden="1" outlineLevel="1">
       <c r="A168" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12206,7 +12218,7 @@
       <c r="X168" s="15" t="n"/>
       <c r="Y168" s="15" t="n"/>
     </row>
-    <row r="169">
+    <row r="169" hidden="1" outlineLevel="1">
       <c r="A169" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12271,7 +12283,7 @@
       <c r="X169" s="15" t="n"/>
       <c r="Y169" s="15" t="n"/>
     </row>
-    <row r="170">
+    <row r="170" hidden="1" outlineLevel="1">
       <c r="A170" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12336,7 +12348,7 @@
       <c r="X170" s="15" t="n"/>
       <c r="Y170" s="15" t="n"/>
     </row>
-    <row r="171">
+    <row r="171" hidden="1" outlineLevel="1">
       <c r="A171" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12466,7 +12478,7 @@
       <c r="X172" s="15" t="n"/>
       <c r="Y172" s="15" t="n"/>
     </row>
-    <row r="173">
+    <row r="173" hidden="1" outlineLevel="1">
       <c r="A173" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12531,7 +12543,7 @@
       <c r="X173" s="15" t="n"/>
       <c r="Y173" s="15" t="n"/>
     </row>
-    <row r="174">
+    <row r="174" hidden="1" outlineLevel="1">
       <c r="A174" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12596,7 +12608,7 @@
       <c r="X174" s="15" t="n"/>
       <c r="Y174" s="15" t="n"/>
     </row>
-    <row r="175">
+    <row r="175" hidden="1" outlineLevel="1">
       <c r="A175" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12661,7 +12673,7 @@
       <c r="X175" s="15" t="n"/>
       <c r="Y175" s="15" t="n"/>
     </row>
-    <row r="176">
+    <row r="176" hidden="1" outlineLevel="1">
       <c r="A176" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12726,7 +12738,7 @@
       <c r="X176" s="15" t="n"/>
       <c r="Y176" s="15" t="n"/>
     </row>
-    <row r="177">
+    <row r="177" hidden="1" outlineLevel="1">
       <c r="A177" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12791,7 +12803,7 @@
       <c r="X177" s="15" t="n"/>
       <c r="Y177" s="15" t="n"/>
     </row>
-    <row r="178">
+    <row r="178" hidden="1" outlineLevel="1">
       <c r="A178" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -12986,7 +12998,7 @@
       <c r="X180" s="15" t="n"/>
       <c r="Y180" s="15" t="n"/>
     </row>
-    <row r="181">
+    <row r="181" hidden="1" outlineLevel="1">
       <c r="A181" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13051,7 +13063,7 @@
       <c r="X181" s="15" t="n"/>
       <c r="Y181" s="15" t="n"/>
     </row>
-    <row r="182">
+    <row r="182" hidden="1" outlineLevel="1">
       <c r="A182" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13116,7 +13128,7 @@
       <c r="X182" s="15" t="n"/>
       <c r="Y182" s="15" t="n"/>
     </row>
-    <row r="183">
+    <row r="183" hidden="1" outlineLevel="1">
       <c r="A183" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13250,7 +13262,7 @@
       <c r="X184" s="15" t="n"/>
       <c r="Y184" s="15" t="n"/>
     </row>
-    <row r="185">
+    <row r="185" hidden="1" outlineLevel="1">
       <c r="A185" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13319,7 +13331,7 @@
       <c r="X185" s="15" t="n"/>
       <c r="Y185" s="15" t="n"/>
     </row>
-    <row r="186">
+    <row r="186" hidden="1" outlineLevel="1">
       <c r="A186" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13388,7 +13400,7 @@
       <c r="X186" s="15" t="n"/>
       <c r="Y186" s="15" t="n"/>
     </row>
-    <row r="187">
+    <row r="187" hidden="1" outlineLevel="1">
       <c r="A187" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13457,7 +13469,7 @@
       <c r="X187" s="15" t="n"/>
       <c r="Y187" s="15" t="n"/>
     </row>
-    <row r="188">
+    <row r="188" hidden="1" outlineLevel="1">
       <c r="A188" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13591,7 +13603,7 @@
       <c r="X189" s="15" t="n"/>
       <c r="Y189" s="15" t="n"/>
     </row>
-    <row r="190">
+    <row r="190" hidden="1" outlineLevel="1">
       <c r="A190" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13656,7 +13668,7 @@
       <c r="X190" s="15" t="n"/>
       <c r="Y190" s="15" t="n"/>
     </row>
-    <row r="191">
+    <row r="191" hidden="1" outlineLevel="1">
       <c r="A191" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13786,7 +13798,7 @@
       <c r="X192" s="15" t="n"/>
       <c r="Y192" s="15" t="n"/>
     </row>
-    <row r="193">
+    <row r="193" hidden="1" outlineLevel="1">
       <c r="A193" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13851,7 +13863,7 @@
       <c r="X193" s="15" t="n"/>
       <c r="Y193" s="15" t="n"/>
     </row>
-    <row r="194">
+    <row r="194" hidden="1" outlineLevel="1">
       <c r="A194" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13916,7 +13928,7 @@
       <c r="X194" s="15" t="n"/>
       <c r="Y194" s="15" t="n"/>
     </row>
-    <row r="195">
+    <row r="195" hidden="1" outlineLevel="1">
       <c r="A195" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -13981,7 +13993,7 @@
       <c r="X195" s="15" t="n"/>
       <c r="Y195" s="15" t="n"/>
     </row>
-    <row r="196">
+    <row r="196" hidden="1" outlineLevel="1">
       <c r="A196" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14046,7 +14058,7 @@
       <c r="X196" s="15" t="n"/>
       <c r="Y196" s="15" t="n"/>
     </row>
-    <row r="197">
+    <row r="197" hidden="1" outlineLevel="1">
       <c r="A197" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14111,7 +14123,7 @@
       <c r="X197" s="15" t="n"/>
       <c r="Y197" s="15" t="n"/>
     </row>
-    <row r="198">
+    <row r="198" hidden="1" outlineLevel="1">
       <c r="A198" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14245,7 +14257,7 @@
       <c r="X199" s="15" t="n"/>
       <c r="Y199" s="15" t="n"/>
     </row>
-    <row r="200">
+    <row r="200" hidden="1" outlineLevel="1">
       <c r="A200" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14314,7 +14326,7 @@
       <c r="X200" s="15" t="n"/>
       <c r="Y200" s="15" t="n"/>
     </row>
-    <row r="201">
+    <row r="201" hidden="1" outlineLevel="1">
       <c r="A201" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14383,7 +14395,7 @@
       <c r="X201" s="15" t="n"/>
       <c r="Y201" s="15" t="n"/>
     </row>
-    <row r="202">
+    <row r="202" hidden="1" outlineLevel="1">
       <c r="A202" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14452,7 +14464,7 @@
       <c r="X202" s="15" t="n"/>
       <c r="Y202" s="15" t="n"/>
     </row>
-    <row r="203">
+    <row r="203" hidden="1" outlineLevel="1">
       <c r="A203" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14586,7 +14598,7 @@
       <c r="X204" s="15" t="n"/>
       <c r="Y204" s="15" t="n"/>
     </row>
-    <row r="205">
+    <row r="205" hidden="1" outlineLevel="1">
       <c r="A205" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14651,7 +14663,7 @@
       <c r="X205" s="15" t="n"/>
       <c r="Y205" s="15" t="n"/>
     </row>
-    <row r="206">
+    <row r="206" hidden="1" outlineLevel="1">
       <c r="A206" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14716,7 +14728,7 @@
       <c r="X206" s="15" t="n"/>
       <c r="Y206" s="15" t="n"/>
     </row>
-    <row r="207">
+    <row r="207" hidden="1" outlineLevel="1">
       <c r="A207" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14781,7 +14793,7 @@
       <c r="X207" s="15" t="n"/>
       <c r="Y207" s="15" t="n"/>
     </row>
-    <row r="208">
+    <row r="208" hidden="1" outlineLevel="1">
       <c r="A208" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14846,7 +14858,7 @@
       <c r="X208" s="15" t="n"/>
       <c r="Y208" s="15" t="n"/>
     </row>
-    <row r="209">
+    <row r="209" hidden="1" outlineLevel="1">
       <c r="A209" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -14911,7 +14923,7 @@
       <c r="X209" s="15" t="n"/>
       <c r="Y209" s="15" t="n"/>
     </row>
-    <row r="210">
+    <row r="210" hidden="1" outlineLevel="1">
       <c r="A210" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15041,7 +15053,7 @@
       <c r="X211" s="15" t="n"/>
       <c r="Y211" s="15" t="n"/>
     </row>
-    <row r="212">
+    <row r="212" hidden="1" outlineLevel="1">
       <c r="A212" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15106,7 +15118,7 @@
       <c r="X212" s="15" t="n"/>
       <c r="Y212" s="15" t="n"/>
     </row>
-    <row r="213">
+    <row r="213" hidden="1" outlineLevel="1">
       <c r="A213" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15171,7 +15183,7 @@
       <c r="X213" s="15" t="n"/>
       <c r="Y213" s="15" t="n"/>
     </row>
-    <row r="214">
+    <row r="214" hidden="1" outlineLevel="1">
       <c r="A214" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15301,7 +15313,7 @@
       <c r="X215" s="15" t="n"/>
       <c r="Y215" s="15" t="n"/>
     </row>
-    <row r="216">
+    <row r="216" hidden="1" outlineLevel="1">
       <c r="A216" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15366,7 +15378,7 @@
       <c r="X216" s="15" t="n"/>
       <c r="Y216" s="15" t="n"/>
     </row>
-    <row r="217">
+    <row r="217" hidden="1" outlineLevel="1">
       <c r="A217" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15496,7 +15508,7 @@
       <c r="X218" s="15" t="n"/>
       <c r="Y218" s="15" t="n"/>
     </row>
-    <row r="219">
+    <row r="219" hidden="1" outlineLevel="1">
       <c r="A219" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15626,7 +15638,7 @@
       <c r="X220" s="15" t="n"/>
       <c r="Y220" s="15" t="n"/>
     </row>
-    <row r="221">
+    <row r="221" hidden="1" outlineLevel="1">
       <c r="A221" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15691,7 +15703,7 @@
       <c r="X221" s="15" t="n"/>
       <c r="Y221" s="15" t="n"/>
     </row>
-    <row r="222">
+    <row r="222" hidden="1" outlineLevel="1">
       <c r="A222" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -15886,7 +15898,7 @@
       <c r="X224" s="15" t="n"/>
       <c r="Y224" s="15" t="n"/>
     </row>
-    <row r="225">
+    <row r="225" hidden="1" outlineLevel="1">
       <c r="A225" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16085,7 +16097,7 @@
       <c r="X227" s="15" t="n"/>
       <c r="Y227" s="15" t="n"/>
     </row>
-    <row r="228">
+    <row r="228" hidden="1" outlineLevel="1">
       <c r="A228" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16219,7 +16231,7 @@
       <c r="X229" s="15" t="n"/>
       <c r="Y229" s="15" t="n"/>
     </row>
-    <row r="230">
+    <row r="230" hidden="1" outlineLevel="1">
       <c r="A230" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16284,7 +16296,7 @@
       <c r="X230" s="15" t="n"/>
       <c r="Y230" s="15" t="n"/>
     </row>
-    <row r="231">
+    <row r="231" hidden="1" outlineLevel="1">
       <c r="A231" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16414,7 +16426,7 @@
       <c r="X232" s="15" t="n"/>
       <c r="Y232" s="15" t="n"/>
     </row>
-    <row r="233">
+    <row r="233" hidden="1" outlineLevel="1">
       <c r="A233" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16479,7 +16491,7 @@
       <c r="X233" s="15" t="n"/>
       <c r="Y233" s="15" t="n"/>
     </row>
-    <row r="234">
+    <row r="234" hidden="1" outlineLevel="1">
       <c r="A234" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16544,7 +16556,7 @@
       <c r="X234" s="15" t="n"/>
       <c r="Y234" s="15" t="n"/>
     </row>
-    <row r="235">
+    <row r="235" hidden="1" outlineLevel="1">
       <c r="A235" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16674,7 +16686,7 @@
       <c r="X236" s="15" t="n"/>
       <c r="Y236" s="15" t="n"/>
     </row>
-    <row r="237">
+    <row r="237" hidden="1" outlineLevel="1">
       <c r="A237" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16739,7 +16751,7 @@
       <c r="X237" s="15" t="n"/>
       <c r="Y237" s="15" t="n"/>
     </row>
-    <row r="238">
+    <row r="238" hidden="1" outlineLevel="1">
       <c r="A238" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16804,7 +16816,7 @@
       <c r="X238" s="15" t="n"/>
       <c r="Y238" s="15" t="n"/>
     </row>
-    <row r="239">
+    <row r="239" hidden="1" outlineLevel="1">
       <c r="A239" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -16934,7 +16946,7 @@
       <c r="X240" s="15" t="n"/>
       <c r="Y240" s="15" t="n"/>
     </row>
-    <row r="241">
+    <row r="241" hidden="1" outlineLevel="1">
       <c r="A241" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -17064,7 +17076,7 @@
       <c r="X242" s="15" t="n"/>
       <c r="Y242" s="15" t="n"/>
     </row>
-    <row r="243">
+    <row r="243" hidden="1" outlineLevel="1">
       <c r="A243" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -17198,7 +17210,7 @@
       <c r="X244" s="15" t="n"/>
       <c r="Y244" s="15" t="n"/>
     </row>
-    <row r="245">
+    <row r="245" hidden="1" outlineLevel="1">
       <c r="A245" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -17267,7 +17279,7 @@
       <c r="X245" s="15" t="n"/>
       <c r="Y245" s="15" t="n"/>
     </row>
-    <row r="246">
+    <row r="246" hidden="1" outlineLevel="1">
       <c r="A246" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -17336,7 +17348,7 @@
       <c r="X246" s="15" t="n"/>
       <c r="Y246" s="15" t="n"/>
     </row>
-    <row r="247">
+    <row r="247" hidden="1" outlineLevel="1">
       <c r="A247" s="9" t="inlineStr">
         <is>
           <t>P1</t>
@@ -17466,7 +17478,7 @@
       <c r="X248" s="15" t="n"/>
       <c r="Y248" s="15" t="n"/>
     </row>
-    <row r="249">
+    <row r="249" hidden="1" outlineLevel="1">
       <c r="A249" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17527,7 +17539,7 @@
       <c r="X249" s="15" t="n"/>
       <c r="Y249" s="15" t="n"/>
     </row>
-    <row r="250">
+    <row r="250" hidden="1" outlineLevel="1">
       <c r="A250" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17588,7 +17600,7 @@
       <c r="X250" s="15" t="n"/>
       <c r="Y250" s="15" t="n"/>
     </row>
-    <row r="251">
+    <row r="251" hidden="1" outlineLevel="1">
       <c r="A251" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17649,7 +17661,7 @@
       <c r="X251" s="15" t="n"/>
       <c r="Y251" s="15" t="n"/>
     </row>
-    <row r="252">
+    <row r="252" hidden="1" outlineLevel="1">
       <c r="A252" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17710,7 +17722,7 @@
       <c r="X252" s="15" t="n"/>
       <c r="Y252" s="15" t="n"/>
     </row>
-    <row r="253">
+    <row r="253" hidden="1" outlineLevel="1">
       <c r="A253" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17836,7 +17848,7 @@
       <c r="X254" s="15" t="n"/>
       <c r="Y254" s="15" t="n"/>
     </row>
-    <row r="255">
+    <row r="255" hidden="1" outlineLevel="1">
       <c r="A255" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17901,7 +17913,7 @@
       <c r="X255" s="15" t="n"/>
       <c r="Y255" s="15" t="n"/>
     </row>
-    <row r="256">
+    <row r="256" hidden="1" outlineLevel="1">
       <c r="A256" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -17966,7 +17978,7 @@
       <c r="X256" s="15" t="n"/>
       <c r="Y256" s="15" t="n"/>
     </row>
-    <row r="257">
+    <row r="257" hidden="1" outlineLevel="1">
       <c r="A257" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18031,7 +18043,7 @@
       <c r="X257" s="15" t="n"/>
       <c r="Y257" s="15" t="n"/>
     </row>
-    <row r="258">
+    <row r="258" hidden="1" outlineLevel="1">
       <c r="A258" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18096,7 +18108,7 @@
       <c r="X258" s="15" t="n"/>
       <c r="Y258" s="15" t="n"/>
     </row>
-    <row r="259">
+    <row r="259" hidden="1" outlineLevel="1">
       <c r="A259" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18161,7 +18173,7 @@
       <c r="X259" s="15" t="n"/>
       <c r="Y259" s="15" t="n"/>
     </row>
-    <row r="260">
+    <row r="260" hidden="1" outlineLevel="1">
       <c r="A260" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18291,7 +18303,7 @@
       <c r="X261" s="15" t="n"/>
       <c r="Y261" s="15" t="n"/>
     </row>
-    <row r="262">
+    <row r="262" hidden="1" outlineLevel="1">
       <c r="A262" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18356,7 +18368,7 @@
       <c r="X262" s="15" t="n"/>
       <c r="Y262" s="15" t="n"/>
     </row>
-    <row r="263">
+    <row r="263" hidden="1" outlineLevel="1">
       <c r="A263" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18421,7 +18433,7 @@
       <c r="X263" s="15" t="n"/>
       <c r="Y263" s="15" t="n"/>
     </row>
-    <row r="264">
+    <row r="264" hidden="1" outlineLevel="1">
       <c r="A264" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18555,7 +18567,7 @@
       <c r="X265" s="15" t="n"/>
       <c r="Y265" s="15" t="n"/>
     </row>
-    <row r="266">
+    <row r="266" hidden="1" outlineLevel="1">
       <c r="A266" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18624,7 +18636,7 @@
       <c r="X266" s="15" t="n"/>
       <c r="Y266" s="15" t="n"/>
     </row>
-    <row r="267">
+    <row r="267" hidden="1" outlineLevel="1">
       <c r="A267" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18693,7 +18705,7 @@
       <c r="X267" s="15" t="n"/>
       <c r="Y267" s="15" t="n"/>
     </row>
-    <row r="268">
+    <row r="268" hidden="1" outlineLevel="1">
       <c r="A268" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18762,7 +18774,7 @@
       <c r="X268" s="15" t="n"/>
       <c r="Y268" s="15" t="n"/>
     </row>
-    <row r="269">
+    <row r="269" hidden="1" outlineLevel="1">
       <c r="A269" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18831,7 +18843,7 @@
       <c r="X269" s="15" t="n"/>
       <c r="Y269" s="15" t="n"/>
     </row>
-    <row r="270">
+    <row r="270" hidden="1" outlineLevel="1">
       <c r="A270" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -18965,7 +18977,7 @@
       <c r="X271" s="15" t="n"/>
       <c r="Y271" s="15" t="n"/>
     </row>
-    <row r="272">
+    <row r="272" hidden="1" outlineLevel="1">
       <c r="A272" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19099,7 +19111,7 @@
       <c r="X273" s="15" t="n"/>
       <c r="Y273" s="15" t="n"/>
     </row>
-    <row r="274">
+    <row r="274" hidden="1" outlineLevel="1">
       <c r="A274" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19168,7 +19180,7 @@
       <c r="X274" s="15" t="n"/>
       <c r="Y274" s="15" t="n"/>
     </row>
-    <row r="275">
+    <row r="275" hidden="1" outlineLevel="1">
       <c r="A275" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19237,7 +19249,7 @@
       <c r="X275" s="15" t="n"/>
       <c r="Y275" s="15" t="n"/>
     </row>
-    <row r="276">
+    <row r="276" hidden="1" outlineLevel="1">
       <c r="A276" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19306,7 +19318,7 @@
       <c r="X276" s="15" t="n"/>
       <c r="Y276" s="15" t="n"/>
     </row>
-    <row r="277">
+    <row r="277" hidden="1" outlineLevel="1">
       <c r="A277" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19444,7 +19456,7 @@
       <c r="X278" s="15" t="n"/>
       <c r="Y278" s="15" t="n"/>
     </row>
-    <row r="279">
+    <row r="279" hidden="1" outlineLevel="1">
       <c r="A279" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19513,7 +19525,7 @@
       <c r="X279" s="15" t="n"/>
       <c r="Y279" s="15" t="n"/>
     </row>
-    <row r="280">
+    <row r="280" hidden="1" outlineLevel="1">
       <c r="A280" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19647,7 +19659,7 @@
       <c r="X281" s="15" t="n"/>
       <c r="Y281" s="15" t="n"/>
     </row>
-    <row r="282">
+    <row r="282" hidden="1" outlineLevel="1">
       <c r="A282" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19712,7 +19724,7 @@
       <c r="X282" s="15" t="n"/>
       <c r="Y282" s="15" t="n"/>
     </row>
-    <row r="283">
+    <row r="283" hidden="1" outlineLevel="1">
       <c r="A283" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19842,7 +19854,7 @@
       <c r="X284" s="15" t="n"/>
       <c r="Y284" s="15" t="n"/>
     </row>
-    <row r="285">
+    <row r="285" hidden="1" outlineLevel="1">
       <c r="A285" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -19972,7 +19984,7 @@
       <c r="X286" s="15" t="n"/>
       <c r="Y286" s="15" t="n"/>
     </row>
-    <row r="287">
+    <row r="287" hidden="1" outlineLevel="1">
       <c r="A287" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20037,7 +20049,7 @@
       <c r="X287" s="15" t="n"/>
       <c r="Y287" s="15" t="n"/>
     </row>
-    <row r="288">
+    <row r="288" hidden="1" outlineLevel="1">
       <c r="A288" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20102,7 +20114,7 @@
       <c r="X288" s="15" t="n"/>
       <c r="Y288" s="15" t="n"/>
     </row>
-    <row r="289">
+    <row r="289" hidden="1" outlineLevel="1">
       <c r="A289" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20167,7 +20179,7 @@
       <c r="X289" s="15" t="n"/>
       <c r="Y289" s="15" t="n"/>
     </row>
-    <row r="290">
+    <row r="290" hidden="1" outlineLevel="1">
       <c r="A290" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20297,7 +20309,7 @@
       <c r="X291" s="15" t="n"/>
       <c r="Y291" s="15" t="n"/>
     </row>
-    <row r="292">
+    <row r="292" hidden="1" outlineLevel="1">
       <c r="A292" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20362,7 +20374,7 @@
       <c r="X292" s="15" t="n"/>
       <c r="Y292" s="15" t="n"/>
     </row>
-    <row r="293">
+    <row r="293" hidden="1" outlineLevel="1">
       <c r="A293" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20427,7 +20439,7 @@
       <c r="X293" s="15" t="n"/>
       <c r="Y293" s="15" t="n"/>
     </row>
-    <row r="294">
+    <row r="294" hidden="1" outlineLevel="1">
       <c r="A294" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20492,7 +20504,7 @@
       <c r="X294" s="15" t="n"/>
       <c r="Y294" s="15" t="n"/>
     </row>
-    <row r="295">
+    <row r="295" hidden="1" outlineLevel="1">
       <c r="A295" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20557,7 +20569,7 @@
       <c r="X295" s="15" t="n"/>
       <c r="Y295" s="15" t="n"/>
     </row>
-    <row r="296">
+    <row r="296" hidden="1" outlineLevel="1">
       <c r="A296" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20622,7 +20634,7 @@
       <c r="X296" s="15" t="n"/>
       <c r="Y296" s="15" t="n"/>
     </row>
-    <row r="297">
+    <row r="297" hidden="1" outlineLevel="1">
       <c r="A297" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20752,7 +20764,7 @@
       <c r="X298" s="15" t="n"/>
       <c r="Y298" s="15" t="n"/>
     </row>
-    <row r="299">
+    <row r="299" hidden="1" outlineLevel="1">
       <c r="A299" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20817,7 +20829,7 @@
       <c r="X299" s="15" t="n"/>
       <c r="Y299" s="15" t="n"/>
     </row>
-    <row r="300">
+    <row r="300" hidden="1" outlineLevel="1">
       <c r="A300" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -20947,7 +20959,7 @@
       <c r="X301" s="15" t="n"/>
       <c r="Y301" s="15" t="n"/>
     </row>
-    <row r="302">
+    <row r="302" hidden="1" outlineLevel="1">
       <c r="A302" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21077,7 +21089,7 @@
       <c r="X303" s="15" t="n"/>
       <c r="Y303" s="15" t="n"/>
     </row>
-    <row r="304">
+    <row r="304" hidden="1" outlineLevel="1">
       <c r="A304" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21211,7 +21223,7 @@
       <c r="X305" s="15" t="n"/>
       <c r="Y305" s="15" t="n"/>
     </row>
-    <row r="306">
+    <row r="306" hidden="1" outlineLevel="1">
       <c r="A306" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21280,7 +21292,7 @@
       <c r="X306" s="15" t="n"/>
       <c r="Y306" s="15" t="n"/>
     </row>
-    <row r="307">
+    <row r="307" hidden="1" outlineLevel="1">
       <c r="A307" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21349,7 +21361,7 @@
       <c r="X307" s="15" t="n"/>
       <c r="Y307" s="15" t="n"/>
     </row>
-    <row r="308">
+    <row r="308" hidden="1" outlineLevel="1">
       <c r="A308" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21418,7 +21430,7 @@
       <c r="X308" s="15" t="n"/>
       <c r="Y308" s="15" t="n"/>
     </row>
-    <row r="309">
+    <row r="309" hidden="1" outlineLevel="1">
       <c r="A309" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21552,7 +21564,7 @@
       <c r="X310" s="15" t="n"/>
       <c r="Y310" s="15" t="n"/>
     </row>
-    <row r="311">
+    <row r="311" hidden="1" outlineLevel="1">
       <c r="A311" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21617,7 +21629,7 @@
       <c r="X311" s="15" t="n"/>
       <c r="Y311" s="15" t="n"/>
     </row>
-    <row r="312">
+    <row r="312" hidden="1" outlineLevel="1">
       <c r="A312" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21682,7 +21694,7 @@
       <c r="X312" s="15" t="n"/>
       <c r="Y312" s="15" t="n"/>
     </row>
-    <row r="313">
+    <row r="313" hidden="1" outlineLevel="1">
       <c r="A313" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21747,7 +21759,7 @@
       <c r="X313" s="15" t="n"/>
       <c r="Y313" s="15" t="n"/>
     </row>
-    <row r="314">
+    <row r="314" hidden="1" outlineLevel="1">
       <c r="A314" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21812,7 +21824,7 @@
       <c r="X314" s="15" t="n"/>
       <c r="Y314" s="15" t="n"/>
     </row>
-    <row r="315">
+    <row r="315" hidden="1" outlineLevel="1">
       <c r="A315" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -21877,7 +21889,7 @@
       <c r="X315" s="15" t="n"/>
       <c r="Y315" s="15" t="n"/>
     </row>
-    <row r="316">
+    <row r="316" hidden="1" outlineLevel="1">
       <c r="A316" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22011,7 +22023,7 @@
       <c r="X317" s="15" t="n"/>
       <c r="Y317" s="15" t="n"/>
     </row>
-    <row r="318">
+    <row r="318" hidden="1" outlineLevel="1">
       <c r="A318" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22080,7 +22092,7 @@
       <c r="X318" s="15" t="n"/>
       <c r="Y318" s="15" t="n"/>
     </row>
-    <row r="319">
+    <row r="319" hidden="1" outlineLevel="1">
       <c r="A319" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22214,7 +22226,7 @@
       <c r="X320" s="15" t="n"/>
       <c r="Y320" s="15" t="n"/>
     </row>
-    <row r="321">
+    <row r="321" hidden="1" outlineLevel="1">
       <c r="A321" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22279,7 +22291,7 @@
       <c r="X321" s="15" t="n"/>
       <c r="Y321" s="15" t="n"/>
     </row>
-    <row r="322">
+    <row r="322" hidden="1" outlineLevel="1">
       <c r="A322" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22344,7 +22356,7 @@
       <c r="X322" s="15" t="n"/>
       <c r="Y322" s="15" t="n"/>
     </row>
-    <row r="323">
+    <row r="323" hidden="1" outlineLevel="1">
       <c r="A323" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22409,7 +22421,7 @@
       <c r="X323" s="15" t="n"/>
       <c r="Y323" s="15" t="n"/>
     </row>
-    <row r="324">
+    <row r="324" hidden="1" outlineLevel="1">
       <c r="A324" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22474,7 +22486,7 @@
       <c r="X324" s="15" t="n"/>
       <c r="Y324" s="15" t="n"/>
     </row>
-    <row r="325">
+    <row r="325" hidden="1" outlineLevel="1">
       <c r="A325" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22669,7 +22681,7 @@
       <c r="X327" s="15" t="n"/>
       <c r="Y327" s="15" t="n"/>
     </row>
-    <row r="328">
+    <row r="328" hidden="1" outlineLevel="1">
       <c r="A328" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22734,7 +22746,7 @@
       <c r="X328" s="15" t="n"/>
       <c r="Y328" s="15" t="n"/>
     </row>
-    <row r="329">
+    <row r="329" hidden="1" outlineLevel="1">
       <c r="A329" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22799,7 +22811,7 @@
       <c r="X329" s="15" t="n"/>
       <c r="Y329" s="15" t="n"/>
     </row>
-    <row r="330">
+    <row r="330" hidden="1" outlineLevel="1">
       <c r="A330" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22929,7 +22941,7 @@
       <c r="X331" s="15" t="n"/>
       <c r="Y331" s="15" t="n"/>
     </row>
-    <row r="332">
+    <row r="332" hidden="1" outlineLevel="1">
       <c r="A332" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -22994,7 +23006,7 @@
       <c r="X332" s="15" t="n"/>
       <c r="Y332" s="15" t="n"/>
     </row>
-    <row r="333">
+    <row r="333" hidden="1" outlineLevel="1">
       <c r="A333" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23128,7 +23140,7 @@
       <c r="X334" s="15" t="n"/>
       <c r="Y334" s="15" t="n"/>
     </row>
-    <row r="335">
+    <row r="335" hidden="1" outlineLevel="1">
       <c r="A335" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23262,7 +23274,7 @@
       <c r="X336" s="15" t="n"/>
       <c r="Y336" s="15" t="n"/>
     </row>
-    <row r="337">
+    <row r="337" hidden="1" outlineLevel="1">
       <c r="A337" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23327,7 +23339,7 @@
       <c r="X337" s="15" t="n"/>
       <c r="Y337" s="15" t="n"/>
     </row>
-    <row r="338">
+    <row r="338" hidden="1" outlineLevel="1">
       <c r="A338" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23392,7 +23404,7 @@
       <c r="X338" s="15" t="n"/>
       <c r="Y338" s="15" t="n"/>
     </row>
-    <row r="339">
+    <row r="339" hidden="1" outlineLevel="1">
       <c r="A339" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23526,7 +23538,7 @@
       <c r="X340" s="15" t="n"/>
       <c r="Y340" s="15" t="n"/>
     </row>
-    <row r="341">
+    <row r="341" hidden="1" outlineLevel="1">
       <c r="A341" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23595,7 +23607,7 @@
       <c r="X341" s="15" t="n"/>
       <c r="Y341" s="15" t="n"/>
     </row>
-    <row r="342">
+    <row r="342" hidden="1" outlineLevel="1">
       <c r="A342" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23729,7 +23741,7 @@
       <c r="X343" s="15" t="n"/>
       <c r="Y343" s="15" t="n"/>
     </row>
-    <row r="344">
+    <row r="344" hidden="1" outlineLevel="1">
       <c r="A344" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23794,7 +23806,7 @@
       <c r="X344" s="15" t="n"/>
       <c r="Y344" s="15" t="n"/>
     </row>
-    <row r="345">
+    <row r="345" hidden="1" outlineLevel="1">
       <c r="A345" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23859,7 +23871,7 @@
       <c r="X345" s="15" t="n"/>
       <c r="Y345" s="15" t="n"/>
     </row>
-    <row r="346">
+    <row r="346" hidden="1" outlineLevel="1">
       <c r="A346" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -23989,7 +24001,7 @@
       <c r="X347" s="15" t="n"/>
       <c r="Y347" s="15" t="n"/>
     </row>
-    <row r="348">
+    <row r="348" hidden="1" outlineLevel="1">
       <c r="A348" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24054,7 +24066,7 @@
       <c r="X348" s="15" t="n"/>
       <c r="Y348" s="15" t="n"/>
     </row>
-    <row r="349">
+    <row r="349" hidden="1" outlineLevel="1">
       <c r="A349" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24184,7 +24196,7 @@
       <c r="X350" s="15" t="n"/>
       <c r="Y350" s="15" t="n"/>
     </row>
-    <row r="351">
+    <row r="351" hidden="1" outlineLevel="1">
       <c r="A351" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24310,7 +24322,7 @@
       <c r="X352" s="15" t="n"/>
       <c r="Y352" s="15" t="n"/>
     </row>
-    <row r="353">
+    <row r="353" hidden="1" outlineLevel="1">
       <c r="A353" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24371,7 +24383,7 @@
       <c r="X353" s="15" t="n"/>
       <c r="Y353" s="15" t="n"/>
     </row>
-    <row r="354">
+    <row r="354" hidden="1" outlineLevel="1">
       <c r="A354" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24566,7 +24578,7 @@
       <c r="X356" s="15" t="n"/>
       <c r="Y356" s="15" t="n"/>
     </row>
-    <row r="357">
+    <row r="357" hidden="1" outlineLevel="1">
       <c r="A357" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24631,7 +24643,7 @@
       <c r="X357" s="15" t="n"/>
       <c r="Y357" s="15" t="n"/>
     </row>
-    <row r="358">
+    <row r="358" hidden="1" outlineLevel="1">
       <c r="A358" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24696,7 +24708,7 @@
       <c r="X358" s="15" t="n"/>
       <c r="Y358" s="15" t="n"/>
     </row>
-    <row r="359">
+    <row r="359" hidden="1" outlineLevel="1">
       <c r="A359" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24826,7 +24838,7 @@
       <c r="X360" s="15" t="n"/>
       <c r="Y360" s="15" t="n"/>
     </row>
-    <row r="361">
+    <row r="361" hidden="1" outlineLevel="1">
       <c r="A361" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -24956,7 +24968,7 @@
       <c r="X362" s="15" t="n"/>
       <c r="Y362" s="15" t="n"/>
     </row>
-    <row r="363">
+    <row r="363" hidden="1" outlineLevel="1">
       <c r="A363" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25021,7 +25033,7 @@
       <c r="X363" s="15" t="n"/>
       <c r="Y363" s="15" t="n"/>
     </row>
-    <row r="364">
+    <row r="364" hidden="1" outlineLevel="1">
       <c r="A364" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25086,7 +25098,7 @@
       <c r="X364" s="15" t="n"/>
       <c r="Y364" s="15" t="n"/>
     </row>
-    <row r="365">
+    <row r="365" hidden="1" outlineLevel="1">
       <c r="A365" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25151,7 +25163,7 @@
       <c r="X365" s="15" t="n"/>
       <c r="Y365" s="15" t="n"/>
     </row>
-    <row r="366">
+    <row r="366" hidden="1" outlineLevel="1">
       <c r="A366" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25216,7 +25228,7 @@
       <c r="X366" s="15" t="n"/>
       <c r="Y366" s="15" t="n"/>
     </row>
-    <row r="367">
+    <row r="367" hidden="1" outlineLevel="1">
       <c r="A367" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25346,7 +25358,7 @@
       <c r="X368" s="15" t="n"/>
       <c r="Y368" s="15" t="n"/>
     </row>
-    <row r="369">
+    <row r="369" hidden="1" outlineLevel="1">
       <c r="A369" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25411,7 +25423,7 @@
       <c r="X369" s="15" t="n"/>
       <c r="Y369" s="15" t="n"/>
     </row>
-    <row r="370">
+    <row r="370" hidden="1" outlineLevel="1">
       <c r="A370" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25537,7 +25549,7 @@
       <c r="X371" s="15" t="n"/>
       <c r="Y371" s="15" t="n"/>
     </row>
-    <row r="372">
+    <row r="372" hidden="1" outlineLevel="1">
       <c r="A372" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25598,7 +25610,7 @@
       <c r="X372" s="15" t="n"/>
       <c r="Y372" s="15" t="n"/>
     </row>
-    <row r="373">
+    <row r="373" hidden="1" outlineLevel="1">
       <c r="A373" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25793,7 +25805,7 @@
       <c r="X375" s="15" t="n"/>
       <c r="Y375" s="15" t="n"/>
     </row>
-    <row r="376">
+    <row r="376" hidden="1" outlineLevel="1">
       <c r="A376" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -25927,7 +25939,7 @@
       <c r="X377" s="15" t="n"/>
       <c r="Y377" s="15" t="n"/>
     </row>
-    <row r="378">
+    <row r="378" hidden="1" outlineLevel="1">
       <c r="A378" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26057,7 +26069,7 @@
       <c r="X379" s="15" t="n"/>
       <c r="Y379" s="15" t="n"/>
     </row>
-    <row r="380">
+    <row r="380" hidden="1" outlineLevel="1">
       <c r="A380" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26191,7 +26203,7 @@
       <c r="X381" s="15" t="n"/>
       <c r="Y381" s="15" t="n"/>
     </row>
-    <row r="382">
+    <row r="382" hidden="1" outlineLevel="1">
       <c r="A382" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26260,7 +26272,7 @@
       <c r="X382" s="15" t="n"/>
       <c r="Y382" s="15" t="n"/>
     </row>
-    <row r="383">
+    <row r="383" hidden="1" outlineLevel="1">
       <c r="A383" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26329,7 +26341,7 @@
       <c r="X383" s="15" t="n"/>
       <c r="Y383" s="15" t="n"/>
     </row>
-    <row r="384">
+    <row r="384" hidden="1" outlineLevel="1">
       <c r="A384" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26463,7 +26475,7 @@
       <c r="X385" s="15" t="n"/>
       <c r="Y385" s="15" t="n"/>
     </row>
-    <row r="386">
+    <row r="386" hidden="1" outlineLevel="1">
       <c r="A386" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26528,7 +26540,7 @@
       <c r="X386" s="15" t="n"/>
       <c r="Y386" s="15" t="n"/>
     </row>
-    <row r="387">
+    <row r="387" hidden="1" outlineLevel="1">
       <c r="A387" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26662,7 +26674,7 @@
       <c r="X388" s="15" t="n"/>
       <c r="Y388" s="15" t="n"/>
     </row>
-    <row r="389">
+    <row r="389" hidden="1" outlineLevel="1">
       <c r="A389" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26731,7 +26743,7 @@
       <c r="X389" s="15" t="n"/>
       <c r="Y389" s="15" t="n"/>
     </row>
-    <row r="390">
+    <row r="390" hidden="1" outlineLevel="1">
       <c r="A390" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26865,7 +26877,7 @@
       <c r="X391" s="15" t="n"/>
       <c r="Y391" s="15" t="n"/>
     </row>
-    <row r="392">
+    <row r="392" hidden="1" outlineLevel="1">
       <c r="A392" s="10" t="inlineStr">
         <is>
           <t>P2</t>
@@ -26999,7 +27011,7 @@
       <c r="X393" s="15" t="n"/>
       <c r="Y393" s="15" t="n"/>
     </row>
-    <row r="394">
+    <row r="394" hidden="1" outlineLevel="1">
       <c r="A394" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27068,7 +27080,7 @@
       <c r="X394" s="15" t="n"/>
       <c r="Y394" s="15" t="n"/>
     </row>
-    <row r="395">
+    <row r="395" hidden="1" outlineLevel="1">
       <c r="A395" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27137,7 +27149,7 @@
       <c r="X395" s="15" t="n"/>
       <c r="Y395" s="15" t="n"/>
     </row>
-    <row r="396">
+    <row r="396" hidden="1" outlineLevel="1">
       <c r="A396" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27206,7 +27218,7 @@
       <c r="X396" s="15" t="n"/>
       <c r="Y396" s="15" t="n"/>
     </row>
-    <row r="397">
+    <row r="397" hidden="1" outlineLevel="1">
       <c r="A397" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27344,7 +27356,7 @@
       <c r="X398" s="15" t="n"/>
       <c r="Y398" s="15" t="n"/>
     </row>
-    <row r="399">
+    <row r="399" hidden="1" outlineLevel="1">
       <c r="A399" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27413,7 +27425,7 @@
       <c r="X399" s="15" t="n"/>
       <c r="Y399" s="15" t="n"/>
     </row>
-    <row r="400">
+    <row r="400" hidden="1" outlineLevel="1">
       <c r="A400" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27547,7 +27559,7 @@
       <c r="X401" s="15" t="n"/>
       <c r="Y401" s="15" t="n"/>
     </row>
-    <row r="402">
+    <row r="402" hidden="1" outlineLevel="1">
       <c r="A402" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27612,7 +27624,7 @@
       <c r="X402" s="15" t="n"/>
       <c r="Y402" s="15" t="n"/>
     </row>
-    <row r="403">
+    <row r="403" hidden="1" outlineLevel="1">
       <c r="A403" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27677,7 +27689,7 @@
       <c r="X403" s="15" t="n"/>
       <c r="Y403" s="15" t="n"/>
     </row>
-    <row r="404">
+    <row r="404" hidden="1" outlineLevel="1">
       <c r="A404" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27742,7 +27754,7 @@
       <c r="X404" s="15" t="n"/>
       <c r="Y404" s="15" t="n"/>
     </row>
-    <row r="405">
+    <row r="405" hidden="1" outlineLevel="1">
       <c r="A405" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27807,7 +27819,7 @@
       <c r="X405" s="15" t="n"/>
       <c r="Y405" s="15" t="n"/>
     </row>
-    <row r="406">
+    <row r="406" hidden="1" outlineLevel="1">
       <c r="A406" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -27937,7 +27949,7 @@
       <c r="X407" s="15" t="n"/>
       <c r="Y407" s="15" t="n"/>
     </row>
-    <row r="408">
+    <row r="408" hidden="1" outlineLevel="1">
       <c r="A408" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28002,7 +28014,7 @@
       <c r="X408" s="15" t="n"/>
       <c r="Y408" s="15" t="n"/>
     </row>
-    <row r="409">
+    <row r="409" hidden="1" outlineLevel="1">
       <c r="A409" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28132,7 +28144,7 @@
       <c r="X410" s="15" t="n"/>
       <c r="Y410" s="15" t="n"/>
     </row>
-    <row r="411">
+    <row r="411" hidden="1" outlineLevel="1">
       <c r="A411" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28327,7 +28339,7 @@
       <c r="X413" s="15" t="n"/>
       <c r="Y413" s="15" t="n"/>
     </row>
-    <row r="414">
+    <row r="414" hidden="1" outlineLevel="1">
       <c r="A414" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28457,7 +28469,7 @@
       <c r="X415" s="15" t="n"/>
       <c r="Y415" s="15" t="n"/>
     </row>
-    <row r="416">
+    <row r="416" hidden="1" outlineLevel="1">
       <c r="A416" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28587,7 +28599,7 @@
       <c r="X417" s="15" t="n"/>
       <c r="Y417" s="15" t="n"/>
     </row>
-    <row r="418">
+    <row r="418" hidden="1" outlineLevel="1">
       <c r="A418" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28652,7 +28664,7 @@
       <c r="X418" s="15" t="n"/>
       <c r="Y418" s="15" t="n"/>
     </row>
-    <row r="419">
+    <row r="419" hidden="1" outlineLevel="1">
       <c r="A419" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28782,7 +28794,7 @@
       <c r="X420" s="15" t="n"/>
       <c r="Y420" s="15" t="n"/>
     </row>
-    <row r="421">
+    <row r="421" hidden="1" outlineLevel="1">
       <c r="A421" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -28981,7 +28993,7 @@
       <c r="X423" s="15" t="n"/>
       <c r="Y423" s="15" t="n"/>
     </row>
-    <row r="424">
+    <row r="424" hidden="1" outlineLevel="1">
       <c r="A424" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29115,7 +29127,7 @@
       <c r="X425" s="15" t="n"/>
       <c r="Y425" s="15" t="n"/>
     </row>
-    <row r="426">
+    <row r="426" hidden="1" outlineLevel="1">
       <c r="A426" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29180,7 +29192,7 @@
       <c r="X426" s="15" t="n"/>
       <c r="Y426" s="15" t="n"/>
     </row>
-    <row r="427">
+    <row r="427" hidden="1" outlineLevel="1">
       <c r="A427" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29310,7 +29322,7 @@
       <c r="X428" s="15" t="n"/>
       <c r="Y428" s="15" t="n"/>
     </row>
-    <row r="429">
+    <row r="429" hidden="1" outlineLevel="1">
       <c r="A429" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29375,7 +29387,7 @@
       <c r="X429" s="15" t="n"/>
       <c r="Y429" s="15" t="n"/>
     </row>
-    <row r="430">
+    <row r="430" hidden="1" outlineLevel="1">
       <c r="A430" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29505,7 +29517,7 @@
       <c r="X431" s="15" t="n"/>
       <c r="Y431" s="15" t="n"/>
     </row>
-    <row r="432">
+    <row r="432" hidden="1" outlineLevel="1">
       <c r="A432" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29570,7 +29582,7 @@
       <c r="X432" s="15" t="n"/>
       <c r="Y432" s="15" t="n"/>
     </row>
-    <row r="433">
+    <row r="433" hidden="1" outlineLevel="1">
       <c r="A433" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29700,7 +29712,7 @@
       <c r="X434" s="15" t="n"/>
       <c r="Y434" s="15" t="n"/>
     </row>
-    <row r="435">
+    <row r="435" hidden="1" outlineLevel="1">
       <c r="A435" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29834,7 +29846,7 @@
       <c r="X436" s="15" t="n"/>
       <c r="Y436" s="15" t="n"/>
     </row>
-    <row r="437">
+    <row r="437" hidden="1" outlineLevel="1">
       <c r="A437" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -29903,7 +29915,7 @@
       <c r="X437" s="15" t="n"/>
       <c r="Y437" s="15" t="n"/>
     </row>
-    <row r="438">
+    <row r="438" hidden="1" outlineLevel="1">
       <c r="A438" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30037,7 +30049,7 @@
       <c r="X439" s="15" t="n"/>
       <c r="Y439" s="15" t="n"/>
     </row>
-    <row r="440">
+    <row r="440" hidden="1" outlineLevel="1">
       <c r="A440" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30102,7 +30114,7 @@
       <c r="X440" s="15" t="n"/>
       <c r="Y440" s="15" t="n"/>
     </row>
-    <row r="441">
+    <row r="441" hidden="1" outlineLevel="1">
       <c r="A441" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30232,7 +30244,7 @@
       <c r="X442" s="15" t="n"/>
       <c r="Y442" s="15" t="n"/>
     </row>
-    <row r="443">
+    <row r="443" hidden="1" outlineLevel="1">
       <c r="A443" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30297,7 +30309,7 @@
       <c r="X443" s="15" t="n"/>
       <c r="Y443" s="15" t="n"/>
     </row>
-    <row r="444">
+    <row r="444" hidden="1" outlineLevel="1">
       <c r="A444" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30362,7 +30374,7 @@
       <c r="X444" s="15" t="n"/>
       <c r="Y444" s="15" t="n"/>
     </row>
-    <row r="445">
+    <row r="445" hidden="1" outlineLevel="1">
       <c r="A445" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30496,7 +30508,7 @@
       <c r="X446" s="15" t="n"/>
       <c r="Y446" s="15" t="n"/>
     </row>
-    <row r="447">
+    <row r="447" hidden="1" outlineLevel="1">
       <c r="A447" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30565,7 +30577,7 @@
       <c r="X447" s="15" t="n"/>
       <c r="Y447" s="15" t="n"/>
     </row>
-    <row r="448">
+    <row r="448" hidden="1" outlineLevel="1">
       <c r="A448" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30699,7 +30711,7 @@
       <c r="X449" s="15" t="n"/>
       <c r="Y449" s="15" t="n"/>
     </row>
-    <row r="450">
+    <row r="450" hidden="1" outlineLevel="1">
       <c r="A450" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -30833,7 +30845,7 @@
       <c r="X451" s="15" t="n"/>
       <c r="Y451" s="15" t="n"/>
     </row>
-    <row r="452">
+    <row r="452" hidden="1" outlineLevel="1">
       <c r="A452" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31036,7 +31048,7 @@
       <c r="X454" s="15" t="n"/>
       <c r="Y454" s="15" t="n"/>
     </row>
-    <row r="455">
+    <row r="455" hidden="1" outlineLevel="1">
       <c r="A455" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31105,7 +31117,7 @@
       <c r="X455" s="15" t="n"/>
       <c r="Y455" s="15" t="n"/>
     </row>
-    <row r="456">
+    <row r="456" hidden="1" outlineLevel="1">
       <c r="A456" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31174,7 +31186,7 @@
       <c r="X456" s="15" t="n"/>
       <c r="Y456" s="15" t="n"/>
     </row>
-    <row r="457">
+    <row r="457" hidden="1" outlineLevel="1">
       <c r="A457" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31308,7 +31320,7 @@
       <c r="X458" s="15" t="n"/>
       <c r="Y458" s="15" t="n"/>
     </row>
-    <row r="459">
+    <row r="459" hidden="1" outlineLevel="1">
       <c r="A459" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31373,7 +31385,7 @@
       <c r="X459" s="15" t="n"/>
       <c r="Y459" s="15" t="n"/>
     </row>
-    <row r="460">
+    <row r="460" hidden="1" outlineLevel="1">
       <c r="A460" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31438,7 +31450,7 @@
       <c r="X460" s="15" t="n"/>
       <c r="Y460" s="15" t="n"/>
     </row>
-    <row r="461">
+    <row r="461" hidden="1" outlineLevel="1">
       <c r="A461" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31568,7 +31580,7 @@
       <c r="X462" s="15" t="n"/>
       <c r="Y462" s="15" t="n"/>
     </row>
-    <row r="463">
+    <row r="463" hidden="1" outlineLevel="1">
       <c r="A463" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31633,7 +31645,7 @@
       <c r="X463" s="15" t="n"/>
       <c r="Y463" s="15" t="n"/>
     </row>
-    <row r="464">
+    <row r="464" hidden="1" outlineLevel="1">
       <c r="A464" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31763,7 +31775,7 @@
       <c r="X465" s="15" t="n"/>
       <c r="Y465" s="15" t="n"/>
     </row>
-    <row r="466">
+    <row r="466" hidden="1" outlineLevel="1">
       <c r="A466" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -31828,7 +31840,7 @@
       <c r="X466" s="15" t="n"/>
       <c r="Y466" s="15" t="n"/>
     </row>
-    <row r="467">
+    <row r="467" hidden="1" outlineLevel="1">
       <c r="A467" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32088,7 +32100,7 @@
       <c r="X470" s="15" t="n"/>
       <c r="Y470" s="15" t="n"/>
     </row>
-    <row r="471">
+    <row r="471" hidden="1" outlineLevel="1">
       <c r="A471" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32218,7 +32230,7 @@
       <c r="X472" s="15" t="n"/>
       <c r="Y472" s="15" t="n"/>
     </row>
-    <row r="473">
+    <row r="473" hidden="1" outlineLevel="1">
       <c r="A473" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32283,7 +32295,7 @@
       <c r="X473" s="15" t="n"/>
       <c r="Y473" s="15" t="n"/>
     </row>
-    <row r="474">
+    <row r="474" hidden="1" outlineLevel="1">
       <c r="A474" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32348,7 +32360,7 @@
       <c r="X474" s="15" t="n"/>
       <c r="Y474" s="15" t="n"/>
     </row>
-    <row r="475">
+    <row r="475" hidden="1" outlineLevel="1">
       <c r="A475" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32543,7 +32555,7 @@
       <c r="X477" s="15" t="n"/>
       <c r="Y477" s="15" t="n"/>
     </row>
-    <row r="478">
+    <row r="478" hidden="1" outlineLevel="1">
       <c r="A478" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32677,7 +32689,7 @@
       <c r="X479" s="15" t="n"/>
       <c r="Y479" s="15" t="n"/>
     </row>
-    <row r="480">
+    <row r="480" hidden="1" outlineLevel="1">
       <c r="A480" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32811,7 +32823,7 @@
       <c r="X481" s="15" t="n"/>
       <c r="Y481" s="15" t="n"/>
     </row>
-    <row r="482">
+    <row r="482" hidden="1" outlineLevel="1">
       <c r="A482" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -32941,7 +32953,7 @@
       <c r="X483" s="15" t="n"/>
       <c r="Y483" s="15" t="n"/>
     </row>
-    <row r="484">
+    <row r="484" hidden="1" outlineLevel="1">
       <c r="A484" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33006,7 +33018,7 @@
       <c r="X484" s="15" t="n"/>
       <c r="Y484" s="15" t="n"/>
     </row>
-    <row r="485">
+    <row r="485" hidden="1" outlineLevel="1">
       <c r="A485" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33071,7 +33083,7 @@
       <c r="X485" s="15" t="n"/>
       <c r="Y485" s="15" t="n"/>
     </row>
-    <row r="486">
+    <row r="486" hidden="1" outlineLevel="1">
       <c r="A486" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33270,7 +33282,7 @@
       <c r="X488" s="15" t="n"/>
       <c r="Y488" s="15" t="n"/>
     </row>
-    <row r="489">
+    <row r="489" hidden="1" outlineLevel="1">
       <c r="A489" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33339,7 +33351,7 @@
       <c r="X489" s="15" t="n"/>
       <c r="Y489" s="15" t="n"/>
     </row>
-    <row r="490">
+    <row r="490" hidden="1" outlineLevel="1">
       <c r="A490" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33408,7 +33420,7 @@
       <c r="X490" s="15" t="n"/>
       <c r="Y490" s="15" t="n"/>
     </row>
-    <row r="491">
+    <row r="491" hidden="1" outlineLevel="1">
       <c r="A491" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33542,7 +33554,7 @@
       <c r="X492" s="15" t="n"/>
       <c r="Y492" s="15" t="n"/>
     </row>
-    <row r="493">
+    <row r="493" hidden="1" outlineLevel="1">
       <c r="A493" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33607,7 +33619,7 @@
       <c r="X493" s="15" t="n"/>
       <c r="Y493" s="15" t="n"/>
     </row>
-    <row r="494">
+    <row r="494" hidden="1" outlineLevel="1">
       <c r="A494" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33737,7 +33749,7 @@
       <c r="X495" s="15" t="n"/>
       <c r="Y495" s="15" t="n"/>
     </row>
-    <row r="496">
+    <row r="496" hidden="1" outlineLevel="1">
       <c r="A496" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33867,7 +33879,7 @@
       <c r="X497" s="15" t="n"/>
       <c r="Y497" s="15" t="n"/>
     </row>
-    <row r="498">
+    <row r="498" hidden="1" outlineLevel="1">
       <c r="A498" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -33932,7 +33944,7 @@
       <c r="X498" s="15" t="n"/>
       <c r="Y498" s="15" t="n"/>
     </row>
-    <row r="499">
+    <row r="499" hidden="1" outlineLevel="1">
       <c r="A499" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34066,7 +34078,7 @@
       <c r="X500" s="15" t="n"/>
       <c r="Y500" s="15" t="n"/>
     </row>
-    <row r="501">
+    <row r="501" hidden="1" outlineLevel="1">
       <c r="A501" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34200,7 +34212,7 @@
       <c r="X502" s="15" t="n"/>
       <c r="Y502" s="15" t="n"/>
     </row>
-    <row r="503">
+    <row r="503" hidden="1" outlineLevel="1">
       <c r="A503" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34334,7 +34346,7 @@
       <c r="X504" s="15" t="n"/>
       <c r="Y504" s="15" t="n"/>
     </row>
-    <row r="505">
+    <row r="505" hidden="1" outlineLevel="1">
       <c r="A505" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34533,7 +34545,7 @@
       <c r="X507" s="15" t="n"/>
       <c r="Y507" s="15" t="n"/>
     </row>
-    <row r="508">
+    <row r="508" hidden="1" outlineLevel="1">
       <c r="A508" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34663,7 +34675,7 @@
       <c r="X509" s="15" t="n"/>
       <c r="Y509" s="15" t="n"/>
     </row>
-    <row r="510">
+    <row r="510" hidden="1" outlineLevel="1">
       <c r="A510" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34793,7 +34805,7 @@
       <c r="X511" s="15" t="n"/>
       <c r="Y511" s="15" t="n"/>
     </row>
-    <row r="512">
+    <row r="512" hidden="1" outlineLevel="1">
       <c r="A512" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -34923,7 +34935,7 @@
       <c r="X513" s="15" t="n"/>
       <c r="Y513" s="15" t="n"/>
     </row>
-    <row r="514">
+    <row r="514" hidden="1" outlineLevel="1">
       <c r="A514" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35053,7 +35065,7 @@
       <c r="X515" s="15" t="n"/>
       <c r="Y515" s="15" t="n"/>
     </row>
-    <row r="516">
+    <row r="516" hidden="1" outlineLevel="1">
       <c r="A516" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35183,7 +35195,7 @@
       <c r="X517" s="15" t="n"/>
       <c r="Y517" s="15" t="n"/>
     </row>
-    <row r="518">
+    <row r="518" hidden="1" outlineLevel="1">
       <c r="A518" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35248,7 +35260,7 @@
       <c r="X518" s="15" t="n"/>
       <c r="Y518" s="15" t="n"/>
     </row>
-    <row r="519">
+    <row r="519" hidden="1" outlineLevel="1">
       <c r="A519" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35378,7 +35390,7 @@
       <c r="X520" s="15" t="n"/>
       <c r="Y520" s="15" t="n"/>
     </row>
-    <row r="521">
+    <row r="521" hidden="1" outlineLevel="1">
       <c r="A521" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35508,7 +35520,7 @@
       <c r="X522" s="15" t="n"/>
       <c r="Y522" s="15" t="n"/>
     </row>
-    <row r="523">
+    <row r="523" hidden="1" outlineLevel="1">
       <c r="A523" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35573,7 +35585,7 @@
       <c r="X523" s="15" t="n"/>
       <c r="Y523" s="15" t="n"/>
     </row>
-    <row r="524">
+    <row r="524" hidden="1" outlineLevel="1">
       <c r="A524" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35638,7 +35650,7 @@
       <c r="X524" s="15" t="n"/>
       <c r="Y524" s="15" t="n"/>
     </row>
-    <row r="525">
+    <row r="525" hidden="1" outlineLevel="1">
       <c r="A525" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -35768,7 +35780,7 @@
       <c r="X526" s="15" t="n"/>
       <c r="Y526" s="15" t="n"/>
     </row>
-    <row r="527">
+    <row r="527" hidden="1" outlineLevel="1">
       <c r="A527" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36028,7 +36040,7 @@
       <c r="X530" s="15" t="n"/>
       <c r="Y530" s="15" t="n"/>
     </row>
-    <row r="531">
+    <row r="531" hidden="1" outlineLevel="1">
       <c r="A531" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36288,7 +36300,7 @@
       <c r="X534" s="15" t="n"/>
       <c r="Y534" s="15" t="n"/>
     </row>
-    <row r="535">
+    <row r="535" hidden="1" outlineLevel="1">
       <c r="A535" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36353,7 +36365,7 @@
       <c r="X535" s="15" t="n"/>
       <c r="Y535" s="15" t="n"/>
     </row>
-    <row r="536">
+    <row r="536" hidden="1" outlineLevel="1">
       <c r="A536" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36418,7 +36430,7 @@
       <c r="X536" s="15" t="n"/>
       <c r="Y536" s="15" t="n"/>
     </row>
-    <row r="537">
+    <row r="537" hidden="1" outlineLevel="1">
       <c r="A537" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36613,7 +36625,7 @@
       <c r="X539" s="15" t="n"/>
       <c r="Y539" s="15" t="n"/>
     </row>
-    <row r="540">
+    <row r="540" hidden="1" outlineLevel="1">
       <c r="A540" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36869,7 +36881,7 @@
       <c r="X543" s="15" t="n"/>
       <c r="Y543" s="15" t="n"/>
     </row>
-    <row r="544">
+    <row r="544" hidden="1" outlineLevel="1">
       <c r="A544" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -36934,7 +36946,7 @@
       <c r="X544" s="15" t="n"/>
       <c r="Y544" s="15" t="n"/>
     </row>
-    <row r="545">
+    <row r="545" hidden="1" outlineLevel="1">
       <c r="A545" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37064,7 +37076,7 @@
       <c r="X546" s="15" t="n"/>
       <c r="Y546" s="15" t="n"/>
     </row>
-    <row r="547">
+    <row r="547" hidden="1" outlineLevel="1">
       <c r="A547" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37129,7 +37141,7 @@
       <c r="X547" s="15" t="n"/>
       <c r="Y547" s="15" t="n"/>
     </row>
-    <row r="548">
+    <row r="548" hidden="1" outlineLevel="1">
       <c r="A548" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37259,7 +37271,7 @@
       <c r="X549" s="15" t="n"/>
       <c r="Y549" s="15" t="n"/>
     </row>
-    <row r="550">
+    <row r="550" hidden="1" outlineLevel="1">
       <c r="A550" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37324,7 +37336,7 @@
       <c r="X550" s="15" t="n"/>
       <c r="Y550" s="15" t="n"/>
     </row>
-    <row r="551">
+    <row r="551" hidden="1" outlineLevel="1">
       <c r="A551" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37450,7 +37462,7 @@
       <c r="X552" s="15" t="n"/>
       <c r="Y552" s="15" t="n"/>
     </row>
-    <row r="553">
+    <row r="553" hidden="1" outlineLevel="1">
       <c r="A553" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37576,7 +37588,7 @@
       <c r="X554" s="15" t="n"/>
       <c r="Y554" s="15" t="n"/>
     </row>
-    <row r="555">
+    <row r="555" hidden="1" outlineLevel="1">
       <c r="A555" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37641,7 +37653,7 @@
       <c r="X555" s="15" t="n"/>
       <c r="Y555" s="15" t="n"/>
     </row>
-    <row r="556">
+    <row r="556" hidden="1" outlineLevel="1">
       <c r="A556" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -37970,7 +37982,7 @@
       <c r="X560" s="15" t="n"/>
       <c r="Y560" s="15" t="n"/>
     </row>
-    <row r="561">
+    <row r="561" hidden="1" outlineLevel="1">
       <c r="A561" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38035,7 +38047,7 @@
       <c r="X561" s="15" t="n"/>
       <c r="Y561" s="15" t="n"/>
     </row>
-    <row r="562">
+    <row r="562" hidden="1" outlineLevel="1">
       <c r="A562" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38100,7 +38112,7 @@
       <c r="X562" s="15" t="n"/>
       <c r="Y562" s="15" t="n"/>
     </row>
-    <row r="563">
+    <row r="563" hidden="1" outlineLevel="1">
       <c r="A563" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38295,7 +38307,7 @@
       <c r="X565" s="15" t="n"/>
       <c r="Y565" s="15" t="n"/>
     </row>
-    <row r="566">
+    <row r="566" hidden="1" outlineLevel="1">
       <c r="A566" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38360,7 +38372,7 @@
       <c r="X566" s="15" t="n"/>
       <c r="Y566" s="15" t="n"/>
     </row>
-    <row r="567">
+    <row r="567" hidden="1" outlineLevel="1">
       <c r="A567" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38490,7 +38502,7 @@
       <c r="X568" s="15" t="n"/>
       <c r="Y568" s="15" t="n"/>
     </row>
-    <row r="569">
+    <row r="569" hidden="1" outlineLevel="1">
       <c r="A569" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38555,7 +38567,7 @@
       <c r="X569" s="15" t="n"/>
       <c r="Y569" s="15" t="n"/>
     </row>
-    <row r="570">
+    <row r="570" hidden="1" outlineLevel="1">
       <c r="A570" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38685,7 +38697,7 @@
       <c r="X571" s="15" t="n"/>
       <c r="Y571" s="15" t="n"/>
     </row>
-    <row r="572">
+    <row r="572" hidden="1" outlineLevel="1">
       <c r="A572" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38750,7 +38762,7 @@
       <c r="X572" s="15" t="n"/>
       <c r="Y572" s="15" t="n"/>
     </row>
-    <row r="573">
+    <row r="573" hidden="1" outlineLevel="1">
       <c r="A573" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38815,7 +38827,7 @@
       <c r="X573" s="15" t="n"/>
       <c r="Y573" s="15" t="n"/>
     </row>
-    <row r="574">
+    <row r="574" hidden="1" outlineLevel="1">
       <c r="A574" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -38880,7 +38892,7 @@
       <c r="X574" s="15" t="n"/>
       <c r="Y574" s="15" t="n"/>
     </row>
-    <row r="575">
+    <row r="575" hidden="1" outlineLevel="1">
       <c r="A575" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39010,7 +39022,7 @@
       <c r="X576" s="15" t="n"/>
       <c r="Y576" s="15" t="n"/>
     </row>
-    <row r="577">
+    <row r="577" hidden="1" outlineLevel="1">
       <c r="A577" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39075,7 +39087,7 @@
       <c r="X577" s="15" t="n"/>
       <c r="Y577" s="15" t="n"/>
     </row>
-    <row r="578">
+    <row r="578" hidden="1" outlineLevel="1">
       <c r="A578" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39140,7 +39152,7 @@
       <c r="X578" s="15" t="n"/>
       <c r="Y578" s="15" t="n"/>
     </row>
-    <row r="579">
+    <row r="579" hidden="1" outlineLevel="1">
       <c r="A579" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39270,7 +39282,7 @@
       <c r="X580" s="15" t="n"/>
       <c r="Y580" s="15" t="n"/>
     </row>
-    <row r="581">
+    <row r="581" hidden="1" outlineLevel="1">
       <c r="A581" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39335,7 +39347,7 @@
       <c r="X581" s="15" t="n"/>
       <c r="Y581" s="15" t="n"/>
     </row>
-    <row r="582">
+    <row r="582" hidden="1" outlineLevel="1">
       <c r="A582" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39530,7 +39542,7 @@
       <c r="X584" s="15" t="n"/>
       <c r="Y584" s="15" t="n"/>
     </row>
-    <row r="585">
+    <row r="585" hidden="1" outlineLevel="1">
       <c r="A585" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39595,7 +39607,7 @@
       <c r="X585" s="15" t="n"/>
       <c r="Y585" s="15" t="n"/>
     </row>
-    <row r="586">
+    <row r="586" hidden="1" outlineLevel="1">
       <c r="A586" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39725,7 +39737,7 @@
       <c r="X587" s="15" t="n"/>
       <c r="Y587" s="15" t="n"/>
     </row>
-    <row r="588">
+    <row r="588" hidden="1" outlineLevel="1">
       <c r="A588" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39855,7 +39867,7 @@
       <c r="X589" s="15" t="n"/>
       <c r="Y589" s="15" t="n"/>
     </row>
-    <row r="590">
+    <row r="590" hidden="1" outlineLevel="1">
       <c r="A590" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39920,7 +39932,7 @@
       <c r="X590" s="15" t="n"/>
       <c r="Y590" s="15" t="n"/>
     </row>
-    <row r="591">
+    <row r="591" hidden="1" outlineLevel="1">
       <c r="A591" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -39985,7 +39997,7 @@
       <c r="X591" s="15" t="n"/>
       <c r="Y591" s="15" t="n"/>
     </row>
-    <row r="592">
+    <row r="592" hidden="1" outlineLevel="1">
       <c r="A592" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40050,7 +40062,7 @@
       <c r="X592" s="15" t="n"/>
       <c r="Y592" s="15" t="n"/>
     </row>
-    <row r="593">
+    <row r="593" hidden="1" outlineLevel="1">
       <c r="A593" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40180,7 +40192,7 @@
       <c r="X594" s="15" t="n"/>
       <c r="Y594" s="15" t="n"/>
     </row>
-    <row r="595">
+    <row r="595" hidden="1" outlineLevel="1">
       <c r="A595" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40367,7 +40379,7 @@
       <c r="X597" s="15" t="n"/>
       <c r="Y597" s="15" t="n"/>
     </row>
-    <row r="598">
+    <row r="598" hidden="1" outlineLevel="1">
       <c r="A598" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40558,7 +40570,7 @@
       <c r="X600" s="15" t="n"/>
       <c r="Y600" s="15" t="n"/>
     </row>
-    <row r="601">
+    <row r="601" hidden="1" outlineLevel="1">
       <c r="A601" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40688,7 +40700,7 @@
       <c r="X602" s="15" t="n"/>
       <c r="Y602" s="15" t="n"/>
     </row>
-    <row r="603">
+    <row r="603" hidden="1" outlineLevel="1">
       <c r="A603" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40818,7 +40830,7 @@
       <c r="X604" s="15" t="n"/>
       <c r="Y604" s="15" t="n"/>
     </row>
-    <row r="605">
+    <row r="605" hidden="1" outlineLevel="1">
       <c r="A605" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -40883,7 +40895,7 @@
       <c r="X605" s="15" t="n"/>
       <c r="Y605" s="15" t="n"/>
     </row>
-    <row r="606">
+    <row r="606" hidden="1" outlineLevel="1">
       <c r="A606" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41017,7 +41029,7 @@
       <c r="X607" s="15" t="n"/>
       <c r="Y607" s="15" t="n"/>
     </row>
-    <row r="608">
+    <row r="608" hidden="1" outlineLevel="1">
       <c r="A608" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41086,7 +41098,7 @@
       <c r="X608" s="15" t="n"/>
       <c r="Y608" s="15" t="n"/>
     </row>
-    <row r="609">
+    <row r="609" hidden="1" outlineLevel="1">
       <c r="A609" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41220,7 +41232,7 @@
       <c r="X610" s="15" t="n"/>
       <c r="Y610" s="15" t="n"/>
     </row>
-    <row r="611">
+    <row r="611" hidden="1" outlineLevel="1">
       <c r="A611" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41350,7 +41362,7 @@
       <c r="X612" s="15" t="n"/>
       <c r="Y612" s="15" t="n"/>
     </row>
-    <row r="613">
+    <row r="613" hidden="1" outlineLevel="1">
       <c r="A613" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41415,7 +41427,7 @@
       <c r="X613" s="15" t="n"/>
       <c r="Y613" s="15" t="n"/>
     </row>
-    <row r="614">
+    <row r="614" hidden="1" outlineLevel="1">
       <c r="A614" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41545,7 +41557,7 @@
       <c r="X615" s="15" t="n"/>
       <c r="Y615" s="15" t="n"/>
     </row>
-    <row r="616">
+    <row r="616" hidden="1" outlineLevel="1">
       <c r="A616" s="10" t="inlineStr">
         <is>
           <t>P3</t>
@@ -41740,7 +41752,7 @@
       <c r="X618" s="15" t="n"/>
       <c r="Y618" s="15" t="n"/>
     </row>
-    <row r="619">
+    <row r="619" hidden="1" outlineLevel="1">
       <c r="A619" s="10" t="inlineStr">
         <is>
           <t>P3</t>

</xml_diff>

<commit_message>
Synka blankett v1.8 (artal for uppfoljningsplan) + nytt CLAUDE.md
blanketter/blankett_forvaltarkunskap_nnk.xlsx ar en referenskopia, se
CLAUDE.md avsnitt 3 - arbetskopian ligger pa G:. CLAUDE.md saknades
tidigare i detta repot, till skillnad fran Lansstyrelsen och natura-2000.
</commit_message>
<xml_diff>
--- a/blanketter/blankett_forvaltarkunskap_nnk.xlsx
+++ b/blanketter/blankett_forvaltarkunskap_nnk.xlsx
@@ -741,7 +741,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.7, 2026-08-27</t>
+          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.8, 2026-08-27</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="84" customHeight="1">
+    <row r="18" ht="112" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>9.</t>
@@ -877,7 +877,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Kolumn K, "Uppföljningsplan (LST, intern)", är nytt sedan version 1.4 — automatiskt hämtat ur länsstyrelsens interna uppföljningsplaner (153 av 628 rader har en träff, 38 objekt totalt). Visar en målindikator för naturtypen (t.ex. "Död ved", "Granens andel av trädskiktet") med länk till källdokumentet på G:. Källan kallas "Bevarandeplaner" i mappstrukturen på G: men innehåller uppföljningsplaner, inte bevarandetillstånd — förväxla inte med kolumn J. Ett stöd inför Vad ska kontrolleras och Metod för kontroll — inget facit.</t>
+          <t>Kolumn K, "Uppföljningsplan (LST, intern)", är nytt sedan version 1.4 — automatiskt hämtat ur länsstyrelsens interna uppföljningsplaner (153 av 628 rader har en träff, 38 objekt totalt). Visar en målindikator för naturtypen (t.ex. "Död ved", "Granens andel av trädskiktet") med länk till källdokumentet på G:. Källan kallas "Bevarandeplaner" i mappstrukturen på G: men innehåller uppföljningsplaner, inte bevarandetillstånd — förväxla inte med kolumn J. Ett stöd inför Vad ska kontrolleras och Metod för kontroll — inget facit. Sedan version 1.8 avslutas texten med dokumentets årtal inom parentes, t.ex. "...(2018)" — samtliga 38 uppföljningsplaner är från 2017 eller 2018, alltså 8–9 år gamla. Fråga alltid förvaltaren om det stämmer fortfarande (se regel R3).</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till)</t>
+          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L48" s="14" t="n"/>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070, 2180)</t>
+          <t>Död ved (9010, 9070, 2180) (2017)</t>
         </is>
       </c>
       <c r="L49" s="14" t="n"/>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L50" s="14" t="n"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+3 till) (2017)</t>
         </is>
       </c>
       <c r="L51" s="14" t="n"/>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L52" s="14" t="n"/>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (1630, 6270, 6510)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (1630, 6270, 6510) (2017)</t>
         </is>
       </c>
       <c r="L53" s="14" t="n"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+3 till) (2017)</t>
         </is>
       </c>
       <c r="L54" s="14" t="n"/>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="K55" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070, 2180)</t>
+          <t>Död ved (9010, 9070, 2180) (2017)</t>
         </is>
       </c>
       <c r="L55" s="14" t="n"/>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="K56" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L56" s="14" t="n"/>
@@ -4809,7 +4809,7 @@
       </c>
       <c r="K57" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L57" s="14" t="n"/>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="K58" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L58" s="14" t="n"/>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="K59" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070, 2180)</t>
+          <t>Död ved (9010, 9070, 2180) (2017)</t>
         </is>
       </c>
       <c r="L59" s="14" t="n"/>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="K60" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L60" s="14" t="n"/>
@@ -5085,7 +5085,7 @@
       </c>
       <c r="K61" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L61" s="14" t="n"/>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="K103" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L103" s="14" t="n"/>
@@ -7888,7 +7888,7 @@
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L104" s="14" t="n"/>
@@ -7957,7 +7957,7 @@
       </c>
       <c r="K105" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L105" s="14" t="n"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L106" s="14" t="n"/>
@@ -8095,7 +8095,7 @@
       </c>
       <c r="K107" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (5130, 6270, 64... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L107" s="14" t="n"/>
@@ -8164,7 +8164,7 @@
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (3 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (3 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L108" s="14" t="n"/>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="K109" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070)</t>
+          <t>Död ved (9010, 9070) (2018)</t>
         </is>
       </c>
       <c r="L109" s="14" t="n"/>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till)</t>
+          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L110" s="14" t="n"/>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="K111" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L111" s="14" t="n"/>
@@ -8440,7 +8440,7 @@
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L112" s="14" t="n"/>
@@ -8509,7 +8509,7 @@
       </c>
       <c r="K113" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L113" s="14" t="n"/>
@@ -8578,7 +8578,7 @@
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L114" s="14" t="n"/>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="K115" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L115" s="14" t="n"/>
@@ -8716,7 +8716,7 @@
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L116" s="14" t="n"/>
@@ -8785,7 +8785,7 @@
       </c>
       <c r="K117" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070)</t>
+          <t>Död ved (9010, 9070) (2018)</t>
         </is>
       </c>
       <c r="L117" s="14" t="n"/>
@@ -8854,7 +8854,7 @@
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6510) (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L118" s="14" t="n"/>
@@ -8923,7 +8923,7 @@
       </c>
       <c r="K119" s="12" t="inlineStr">
         <is>
-          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till)</t>
+          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (6270, 6510, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L119" s="14" t="n"/>
@@ -8992,7 +8992,7 @@
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L120" s="14" t="n"/>
@@ -9061,7 +9061,7 @@
       </c>
       <c r="K121" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L121" s="14" t="n"/>
@@ -9520,7 +9520,7 @@
       </c>
       <c r="K128" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9070)</t>
+          <t>Död ved (9010, 9070) (2018)</t>
         </is>
       </c>
       <c r="L128" s="14" t="n"/>
@@ -9589,7 +9589,7 @@
       </c>
       <c r="K129" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L129" s="14" t="n"/>
@@ -9658,7 +9658,7 @@
       </c>
       <c r="K130" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (1620, 1630, 6270, 8230, 9070)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (1620, 1630, 6270, 8230, 9070) (2018)</t>
         </is>
       </c>
       <c r="L130" s="14" t="n"/>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="K131" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L131" s="14" t="n"/>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="K132" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L132" s="14" t="n"/>
@@ -9865,7 +9865,7 @@
       </c>
       <c r="K133" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6270, 82... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L133" s="14" t="n"/>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="K134" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L134" s="14" t="n"/>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="K135" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L135" s="14" t="n"/>
@@ -10072,7 +10072,7 @@
       </c>
       <c r="K136" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L136" s="14" t="n"/>
@@ -10401,7 +10401,7 @@
       </c>
       <c r="K141" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L141" s="14" t="n"/>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="K142" s="12" t="inlineStr">
         <is>
-          <t>Det ska finna tillräckligt inslag av död ved (9010, 9050)</t>
+          <t>Det ska finna tillräckligt inslag av död ved (9010, 9050) (2017)</t>
         </is>
       </c>
       <c r="L142" s="14" t="n"/>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="K143" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L143" s="14" t="n"/>
@@ -10608,7 +10608,7 @@
       </c>
       <c r="K144" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070)</t>
+          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070) (2017)</t>
         </is>
       </c>
       <c r="L144" s="14" t="n"/>
@@ -10677,7 +10677,7 @@
       </c>
       <c r="K145" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070)</t>
+          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070) (2017)</t>
         </is>
       </c>
       <c r="L145" s="14" t="n"/>
@@ -10746,7 +10746,7 @@
       </c>
       <c r="K146" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L146" s="14" t="n"/>
@@ -10815,7 +10815,7 @@
       </c>
       <c r="K147" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070)</t>
+          <t>Inslaget av igenväxningsvegetation ska vara mycket begränsat (9070) (2017)</t>
         </is>
       </c>
       <c r="L147" s="14" t="n"/>
@@ -10884,7 +10884,7 @@
       </c>
       <c r="K148" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (8 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L148" s="14" t="n"/>
@@ -11668,7 +11668,7 @@
       </c>
       <c r="K160" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L160" s="14" t="n"/>
@@ -11737,7 +11737,7 @@
       </c>
       <c r="K161" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L161" s="14" t="n"/>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="K162" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L162" s="14" t="n"/>
@@ -11875,7 +11875,7 @@
       </c>
       <c r="K163" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L163" s="14" t="n"/>
@@ -11944,7 +11944,7 @@
       </c>
       <c r="K164" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L164" s="14" t="n"/>
@@ -12013,7 +12013,7 @@
       </c>
       <c r="K165" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L165" s="14" t="n"/>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="K166" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6410, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L166" s="14" t="n"/>
@@ -13256,7 +13256,7 @@
       </c>
       <c r="K184" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L184" s="14" t="n"/>
@@ -13325,7 +13325,7 @@
       </c>
       <c r="K185" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L185" s="14" t="n"/>
@@ -13394,7 +13394,7 @@
       </c>
       <c r="K186" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L186" s="14" t="n"/>
@@ -13463,7 +13463,7 @@
       </c>
       <c r="K187" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L187" s="14" t="n"/>
@@ -13532,7 +13532,7 @@
       </c>
       <c r="K188" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (1630, 6230, 62... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L188" s="14" t="n"/>
@@ -14251,7 +14251,7 @@
       </c>
       <c r="K199" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L199" s="14" t="n"/>
@@ -14320,7 +14320,7 @@
       </c>
       <c r="K200" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2018)</t>
         </is>
       </c>
       <c r="L200" s="14" t="n"/>
@@ -14389,7 +14389,7 @@
       </c>
       <c r="K201" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2018)</t>
         </is>
       </c>
       <c r="L201" s="14" t="n"/>
@@ -14458,7 +14458,7 @@
       </c>
       <c r="K202" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L202" s="14" t="n"/>
@@ -14527,7 +14527,7 @@
       </c>
       <c r="K203" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L203" s="14" t="n"/>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="K227" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6280) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6280) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L227" s="14" t="n"/>
@@ -16160,7 +16160,7 @@
       </c>
       <c r="K228" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd samt även idegran för...</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd samt även idegran för... (2018)</t>
         </is>
       </c>
       <c r="L228" s="14" t="n"/>
@@ -17204,7 +17204,7 @@
       </c>
       <c r="K244" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9080)</t>
+          <t>Död ved (9010, 9080) (2018)</t>
         </is>
       </c>
       <c r="L244" s="14" t="n"/>
@@ -17273,7 +17273,7 @@
       </c>
       <c r="K245" s="12" t="inlineStr">
         <is>
-          <t>Negativa indikatorarter (7230)</t>
+          <t>Negativa indikatorarter (7230) (2018)</t>
         </is>
       </c>
       <c r="L245" s="14" t="n"/>
@@ -17342,7 +17342,7 @@
       </c>
       <c r="K246" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i lövs... (+1 till)</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i lövs... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L246" s="14" t="n"/>
@@ -17411,7 +17411,7 @@
       </c>
       <c r="K247" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut (1630) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut (1630) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L247" s="14" t="n"/>
@@ -18561,7 +18561,7 @@
       </c>
       <c r="K265" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L265" s="14" t="n"/>
@@ -18630,7 +18630,7 @@
       </c>
       <c r="K266" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut (9070) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut (9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L266" s="14" t="n"/>
@@ -18699,7 +18699,7 @@
       </c>
       <c r="K267" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L267" s="14" t="n"/>
@@ -18768,7 +18768,7 @@
       </c>
       <c r="K268" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L268" s="14" t="n"/>
@@ -18837,7 +18837,7 @@
       </c>
       <c r="K269" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L269" s="14" t="n"/>
@@ -18906,7 +18906,7 @@
       </c>
       <c r="K270" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L270" s="14" t="n"/>
@@ -19105,7 +19105,7 @@
       </c>
       <c r="K273" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L273" s="14" t="n"/>
@@ -19174,7 +19174,7 @@
       </c>
       <c r="K274" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L274" s="14" t="n"/>
@@ -19243,7 +19243,7 @@
       </c>
       <c r="K275" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (5 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L275" s="14" t="n"/>
@@ -19312,7 +19312,7 @@
       </c>
       <c r="K276" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2017)</t>
         </is>
       </c>
       <c r="L276" s="14" t="n"/>
@@ -19381,7 +19381,7 @@
       </c>
       <c r="K277" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2017)</t>
         </is>
       </c>
       <c r="L277" s="14" t="n"/>
@@ -19450,7 +19450,7 @@
       </c>
       <c r="K278" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2018)</t>
         </is>
       </c>
       <c r="L278" s="14" t="n"/>
@@ -19519,7 +19519,7 @@
       </c>
       <c r="K279" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L279" s="14" t="n"/>
@@ -19588,7 +19588,7 @@
       </c>
       <c r="K280" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i eksk... (2018)</t>
         </is>
       </c>
       <c r="L280" s="14" t="n"/>
@@ -21217,7 +21217,7 @@
       </c>
       <c r="K305" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall och triviallövträd för att bestånden ska ... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall och triviallövträd för att bestånden ska ... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L305" s="14" t="n"/>
@@ -21286,7 +21286,7 @@
       </c>
       <c r="K306" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L306" s="14" t="n"/>
@@ -21355,7 +21355,7 @@
       </c>
       <c r="K307" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L307" s="14" t="n"/>
@@ -21424,7 +21424,7 @@
       </c>
       <c r="K308" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i taig...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i taig... (2018)</t>
         </is>
       </c>
       <c r="L308" s="14" t="n"/>
@@ -21493,7 +21493,7 @@
       </c>
       <c r="K309" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L309" s="14" t="n"/>
@@ -22017,7 +22017,7 @@
       </c>
       <c r="K317" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska vara begränsat så att död ved och grova tallar ska vara fortsatt s... (+1 till)</t>
+          <t>Inslaget av gran ska vara begränsat så att död ved och grova tallar ska vara fortsatt s... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L317" s="14" t="n"/>
@@ -22086,7 +22086,7 @@
       </c>
       <c r="K318" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (9 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (9 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L318" s="14" t="n"/>
@@ -22155,7 +22155,7 @@
       </c>
       <c r="K319" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (9 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (9 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L319" s="14" t="n"/>
@@ -23134,7 +23134,7 @@
       </c>
       <c r="K334" s="12" t="inlineStr">
         <is>
-          <t>Brandsubstrat för brandgynnade arter. (9010) (+1 till)</t>
+          <t>Brandsubstrat för brandgynnade arter. (9010) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L334" s="14" t="n"/>
@@ -23203,7 +23203,7 @@
       </c>
       <c r="K335" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L335" s="14" t="n"/>
@@ -23532,7 +23532,7 @@
       </c>
       <c r="K340" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att långsiktigt b... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L340" s="14" t="n"/>
@@ -23601,7 +23601,7 @@
       </c>
       <c r="K341" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L341" s="14" t="n"/>
@@ -23670,7 +23670,7 @@
       </c>
       <c r="K342" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2018)</t>
         </is>
       </c>
       <c r="L342" s="14" t="n"/>
@@ -24507,7 +24507,7 @@
       </c>
       <c r="K355" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall och triviallövträd för att långsiktigt bi... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall och triviallövträd för att långsiktigt bi... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L355" s="14" t="n"/>
@@ -25799,7 +25799,7 @@
       </c>
       <c r="K375" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (3 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (3 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L375" s="14" t="n"/>
@@ -25868,7 +25868,7 @@
       </c>
       <c r="K376" s="12" t="inlineStr">
         <is>
-          <t>Vidkroniga grova träd som tidigare stått ljusöppet ska stå fria i kronan (9160)</t>
+          <t>Vidkroniga grova träd som tidigare stått ljusöppet ska stå fria i kronan (9160) (2017)</t>
         </is>
       </c>
       <c r="L376" s="14" t="n"/>
@@ -26197,7 +26197,7 @@
       </c>
       <c r="K381" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall- och triviallövträd för att bestånden ska... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L381" s="14" t="n"/>
@@ -26266,7 +26266,7 @@
       </c>
       <c r="K382" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i lövs...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i lövs... (2017)</t>
         </is>
       </c>
       <c r="L382" s="14" t="n"/>
@@ -26335,7 +26335,7 @@
       </c>
       <c r="K383" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L383" s="14" t="n"/>
@@ -26404,7 +26404,7 @@
       </c>
       <c r="K384" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (6 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L384" s="14" t="n"/>
@@ -26668,7 +26668,7 @@
       </c>
       <c r="K388" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L388" s="14" t="n"/>
@@ -26737,7 +26737,7 @@
       </c>
       <c r="K389" s="12" t="inlineStr">
         <is>
-          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i taig...</t>
+          <t>Inslaget av gran ska inte påverka artsammansättning eller konkurrensförhållanden i taig... (2017)</t>
         </is>
       </c>
       <c r="L389" s="14" t="n"/>
@@ -26806,7 +26806,7 @@
       </c>
       <c r="K390" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L390" s="14" t="n"/>
@@ -27005,7 +27005,7 @@
       </c>
       <c r="K393" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+3 till) (2017)</t>
         </is>
       </c>
       <c r="L393" s="14" t="n"/>
@@ -27074,7 +27074,7 @@
       </c>
       <c r="K394" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+3 till) (2017)</t>
         </is>
       </c>
       <c r="L394" s="14" t="n"/>
@@ -27143,7 +27143,7 @@
       </c>
       <c r="K395" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9020, 9070)</t>
+          <t>Död ved (9020, 9070) (2017)</t>
         </is>
       </c>
       <c r="L395" s="14" t="n"/>
@@ -27212,7 +27212,7 @@
       </c>
       <c r="K396" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 6410, 8230, 9070)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 6410, 8230, 9070) (2017)</t>
         </is>
       </c>
       <c r="L396" s="14" t="n"/>
@@ -27281,7 +27281,7 @@
       </c>
       <c r="K397" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410, 9070) (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L397" s="14" t="n"/>
@@ -27350,7 +27350,7 @@
       </c>
       <c r="K398" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till) (2018)</t>
         </is>
       </c>
       <c r="L398" s="14" t="n"/>
@@ -27419,7 +27419,7 @@
       </c>
       <c r="K399" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till) (2018)</t>
         </is>
       </c>
       <c r="L399" s="14" t="n"/>
@@ -27488,7 +27488,7 @@
       </c>
       <c r="K400" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+3 till) (2018)</t>
         </is>
       </c>
       <c r="L400" s="14" t="n"/>
@@ -28987,7 +28987,7 @@
       </c>
       <c r="K423" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (9070) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L423" s="14" t="n"/>
@@ -29056,7 +29056,7 @@
       </c>
       <c r="K424" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (8230, 9070)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (8230, 9070) (2018)</t>
         </is>
       </c>
       <c r="L424" s="14" t="n"/>
@@ -29840,7 +29840,7 @@
       </c>
       <c r="K436" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L436" s="14" t="n"/>
@@ -29909,7 +29909,7 @@
       </c>
       <c r="K437" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L437" s="14" t="n"/>
@@ -29978,7 +29978,7 @@
       </c>
       <c r="K438" s="12" t="inlineStr">
         <is>
-          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (silikatgräsmark ...</t>
+          <t>Rödlistade ängs- och hagmarksväxter ska finnas i livskraftiga bestånd (silikatgräsmark ... (2017)</t>
         </is>
       </c>
       <c r="L438" s="14" t="n"/>
@@ -30502,7 +30502,7 @@
       </c>
       <c r="K446" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L446" s="14" t="n"/>
@@ -30571,7 +30571,7 @@
       </c>
       <c r="K447" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L447" s="14" t="n"/>
@@ -30640,7 +30640,7 @@
       </c>
       <c r="K448" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6230, 6270, 6410) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L448" s="14" t="n"/>
@@ -30839,7 +30839,7 @@
       </c>
       <c r="K451" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410) (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410) (+2 till) (2017)</t>
         </is>
       </c>
       <c r="L451" s="14" t="n"/>
@@ -30908,7 +30908,7 @@
       </c>
       <c r="K452" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410) (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (6270, 6410) (+2 till) (2017)</t>
         </is>
       </c>
       <c r="L452" s="14" t="n"/>
@@ -31042,7 +31042,7 @@
       </c>
       <c r="K454" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L454" s="14" t="n"/>
@@ -31111,7 +31111,7 @@
       </c>
       <c r="K455" s="12" t="inlineStr">
         <is>
-          <t>Död ved i olika stadier av nedbrytning och former, såsom lågor, torrakor, högstubbar, h...</t>
+          <t>Död ved i olika stadier av nedbrytning och former, såsom lågor, torrakor, högstubbar, h... (2018)</t>
         </is>
       </c>
       <c r="L455" s="14" t="n"/>
@@ -31180,7 +31180,7 @@
       </c>
       <c r="K456" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd och/eller triviallövträd för att l... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L456" s="14" t="n"/>
@@ -31249,7 +31249,7 @@
       </c>
       <c r="K457" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (6270, 9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L457" s="14" t="n"/>
@@ -32094,7 +32094,7 @@
       </c>
       <c r="K470" s="12" t="inlineStr">
         <is>
-          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (9070) (+1 till)</t>
+          <t>Förekomst av igenväxningsvegetation ska vara mkt begränsad (9070) (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L470" s="14" t="n"/>
@@ -32159,7 +32159,7 @@
       </c>
       <c r="K471" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädellövträd för att långsiktigt bibehålla dess... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädellövträd för att långsiktigt bibehålla dess... (+1 till) (2018)</t>
         </is>
       </c>
       <c r="L471" s="14" t="n"/>
@@ -32683,7 +32683,7 @@
       </c>
       <c r="K479" s="12" t="inlineStr">
         <is>
-          <t>Gran ska inte konkurrera ut lövträd, tall eller naturvårdsträd. (9070) (+2 till)</t>
+          <t>Gran ska inte konkurrera ut lövträd, tall eller naturvårdsträd. (9070) (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L479" s="14" t="n"/>
@@ -32752,7 +32752,7 @@
       </c>
       <c r="K480" s="12" t="inlineStr">
         <is>
-          <t>Igenväxningsvegetation ska inte konkurrera ut typiska arter i området. (6110, 9070) (+2 till)</t>
+          <t>Igenväxningsvegetation ska inte konkurrera ut typiska arter i området. (6110, 9070) (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L480" s="14" t="n"/>
@@ -33276,7 +33276,7 @@
       </c>
       <c r="K488" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+2 till) (2017)</t>
         </is>
       </c>
       <c r="L488" s="14" t="n"/>
@@ -33345,7 +33345,7 @@
       </c>
       <c r="K489" s="12" t="inlineStr">
         <is>
-          <t>Död ved (9010, 9050, 9080)</t>
+          <t>Död ved (9010, 9050, 9080) (2017)</t>
         </is>
       </c>
       <c r="L489" s="14" t="n"/>
@@ -33414,7 +33414,7 @@
       </c>
       <c r="K490" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av ädel- och triviallövträd för att bestånden ska... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L490" s="14" t="n"/>
@@ -33483,7 +33483,7 @@
       </c>
       <c r="K491" s="12" t="inlineStr">
         <is>
-          <t>Igenväxning av öppna myrhabitat (7230) (+1 till)</t>
+          <t>Igenväxning av öppna myrhabitat (7230) (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L491" s="14" t="n"/>
@@ -34072,7 +34072,7 @@
       </c>
       <c r="K500" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L500" s="14" t="n"/>
@@ -34141,7 +34141,7 @@
       </c>
       <c r="K501" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (4 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L501" s="14" t="n"/>
@@ -34340,7 +34340,7 @@
       </c>
       <c r="K504" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall och ädellövträd för att långsiktigt bibeh... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall och ädellövträd för att långsiktigt bibeh... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L504" s="14" t="n"/>
@@ -34409,7 +34409,7 @@
       </c>
       <c r="K505" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av tall och ädellövträd för att långsiktigt bibeh... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av tall och ädellövträd för att långsiktigt bibeh... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L505" s="14" t="n"/>
@@ -35514,7 +35514,7 @@
       </c>
       <c r="K522" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L522" s="14" t="n"/>
@@ -35579,7 +35579,7 @@
       </c>
       <c r="K523" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L523" s="14" t="n"/>
@@ -35644,7 +35644,7 @@
       </c>
       <c r="K524" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L524" s="14" t="n"/>
@@ -35709,7 +35709,7 @@
       </c>
       <c r="K525" s="12" t="inlineStr">
         <is>
-          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod)</t>
+          <t>Uppföljningsplan finns för objektet (2 indikatorer, ej för denna kod) (2017)</t>
         </is>
       </c>
       <c r="L525" s="14" t="n"/>
@@ -37781,7 +37781,7 @@
       </c>
       <c r="K557" s="12" t="inlineStr">
         <is>
-          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (kalkgräsmark (... (+2 till)</t>
+          <t>Grässvålen ska vara väl avbetad/avslagen vid vegetationsperiodens slut. (kalkgräsmark (... (+2 till) (2017)</t>
         </is>
       </c>
       <c r="L557" s="14" t="n"/>
@@ -41023,7 +41023,7 @@
       </c>
       <c r="K607" s="12" t="inlineStr">
         <is>
-          <t>Död ved i olika stadier av nedbrytning och former, såsom lågor, torrakor, högstubbar oc...</t>
+          <t>Död ved i olika stadier av nedbrytning och former, såsom lågor, torrakor, högstubbar oc... (2018)</t>
         </is>
       </c>
       <c r="L607" s="14" t="n"/>
@@ -41092,7 +41092,7 @@
       </c>
       <c r="K608" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av lövträd och/eller tall i områden där dessa trä... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av lövträd och/eller tall i områden där dessa trä... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L608" s="14" t="n"/>
@@ -41161,7 +41161,7 @@
       </c>
       <c r="K609" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av lövträd och/eller tall i områden där dessa trä... (+2 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av lövträd och/eller tall i områden där dessa trä... (+2 till) (2018)</t>
         </is>
       </c>
       <c r="L609" s="14" t="n"/>
@@ -42396,7 +42396,7 @@
       </c>
       <c r="K628" s="12" t="inlineStr">
         <is>
-          <t>Det ska finnas tillräcklig föryngring av triviallövträd för att bestånden ska bestå gen... (+1 till)</t>
+          <t>Det ska finnas tillräcklig föryngring av triviallövträd för att bestånden ska bestå gen... (+1 till) (2017)</t>
         </is>
       </c>
       <c r="L628" s="14" t="n"/>

</xml_diff>